<commit_message>
feat(acm): 132 v4 — area construida 196 m2 + lente de terreno (~220 m2 provisorio)
- Area construida oficial = 196 m2 (era 220 estimado): lente de construcao Top5 = R$ 1.773.948

- Lente de TERRENO ativada como leitura independente: ~220 m2 x R$9.000/m2 terreno = ~R$1.980.000 -> duas lentes formam faixa R$1,77-1,98M; anuncio 18,7% abaixo (subprecificacao mantida)

- DECISAO METODOLOGICA: terreno NAO entra no ranking de aderencia (colapsaria a mediana de construcao com casas terreno-similares baratas/ITBI subdeclarado — artefato R$1,27M). Documentado no codigo + ROADMAP 10.4

- Caveat: 6 vagas em lote ~220 m2 e apertado (CA~0,9) -> terreno pode ser maior (condicionante n1)

- XLSX rev3 self-check Top3 = Juruena 87 / Pariquera-Acu 41 / TV Sebastiao Emilio Forli 58 CONFERE; typecheck+eslint limpos

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/acm/andrade-pertence-132/ACM-AndradePertence132-validacao-corretor-rev3.xlsx
+++ b/docs/acm/andrade-pertence-132/ACM-AndradePertence132-validacao-corretor-rev3.xlsx
@@ -433,7 +433,7 @@
         <v>Programa do alvo</v>
       </c>
       <c r="B3" t="str">
-        <v>220 m² constr. (anúncios divergem 196–220 — confirmar) · terreno NÃO informado · 4 quartos (2 suítes) · 6 vagas · conservado — pronto para morar (apresentação)</v>
+        <v>196 m² constr. (anúncios divergem 196–220 — confirmar) · terreno NÃO informado · 4 quartos (2 suítes) · 6 vagas · conservado — pronto para morar (apresentação)</v>
       </c>
     </row>
     <row r="4">
@@ -565,7 +565,7 @@
         <v>ORDENAÇÃO</v>
       </c>
       <c r="B21" t="str">
-        <v>Ranking por ADERÊNCIA da metodologia: área construída (50%) + área terreno (20% — inerte só pelo lado do alvo: metragem não informada) + proximidade (30%). Top 3 = R UBAIRA 60 · R JURUENA 87 · R PARIQUERA-ACU 41.</v>
+        <v>Ranking por ADERÊNCIA da metodologia: área construída (50%) + área terreno (20% — inerte só pelo lado do alvo: metragem não informada) + proximidade (30%). Top 3 = R JURUENA 87 · R PARIQUERA-ACU 41 · TV SEBASTIAO EMILIO FORLI 58.</v>
       </c>
     </row>
     <row r="22">
@@ -694,7 +694,7 @@
         <v>Gerado em</v>
       </c>
       <c r="B39" t="str">
-        <v>09/07/2026, 07:20:10</v>
+        <v>09/07/2026, 16:02:24</v>
       </c>
     </row>
   </sheetData>
@@ -789,40 +789,40 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>R UBAIRA 60</v>
+        <v>R JURUENA 87</v>
       </c>
       <c r="C2" t="str">
         <v>Moema</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-08</v>
+        <v>2024-11</v>
       </c>
       <c r="E2" t="str">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="F2" t="str">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G2" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H2" t="str">
-        <v>R$ 3.400.000</v>
+        <v>R$ 1.800.000</v>
       </c>
       <c r="I2" t="str">
-        <v>13.600</v>
+        <v>10.000</v>
       </c>
       <c r="J2" t="str">
-        <v>1.0288</v>
+        <v>1.0648</v>
       </c>
       <c r="K2" t="str">
-        <v>13.991</v>
+        <v>10.648</v>
       </c>
       <c r="L2" t="str">
-        <v>4117200224</v>
+        <v>4117200100</v>
       </c>
       <c r="M2" t="str">
-        <v>~282 m (geocode da base)</v>
+        <v>~272 m (geocode da base)</v>
       </c>
       <c r="N2" t="str">
         <v>Abrir no Maps</v>
@@ -845,40 +845,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>R JURUENA 87</v>
+        <v>R PARIQUERA-ACU 41</v>
       </c>
       <c r="C3" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D3" t="str">
-        <v>2024-11</v>
+        <v>2026-03</v>
       </c>
       <c r="E3" t="str">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="F3" t="str">
-        <v>303</v>
+        <v>—</v>
       </c>
       <c r="G3" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H3" t="str">
-        <v>R$ 1.800.000</v>
+        <v>R$ 2.500.000</v>
       </c>
       <c r="I3" t="str">
-        <v>10.000</v>
+        <v>12.438</v>
       </c>
       <c r="J3" t="str">
-        <v>1.0648</v>
+        <v>1.0050</v>
       </c>
       <c r="K3" t="str">
-        <v>10.648</v>
+        <v>12.500</v>
       </c>
       <c r="L3" t="str">
-        <v>4117200100</v>
+        <v>4115400234</v>
       </c>
       <c r="M3" t="str">
-        <v>~272 m (geocode da base)</v>
+        <v>~441 m (geocode da base)</v>
       </c>
       <c r="N3" t="str">
         <v>Abrir no Maps</v>
@@ -893,7 +893,7 @@
         <v/>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="4">
@@ -901,40 +901,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>R PARIQUERA-ACU 41</v>
+        <v>TV SEBASTIAO EMILIO FORLI 58</v>
       </c>
       <c r="C4" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-03</v>
+        <v>2024-05</v>
       </c>
       <c r="E4" t="str">
-        <v>201</v>
+        <v>177</v>
       </c>
       <c r="F4" t="str">
-        <v>—</v>
+        <v>116</v>
       </c>
       <c r="G4" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H4" t="str">
-        <v>R$ 2.500.000</v>
+        <v>R$ 2.900.000</v>
       </c>
       <c r="I4" t="str">
-        <v>12.438</v>
+        <v>16.384</v>
       </c>
       <c r="J4" t="str">
-        <v>1.0050</v>
+        <v>1.1019</v>
       </c>
       <c r="K4" t="str">
-        <v>12.500</v>
+        <v>18.054</v>
       </c>
       <c r="L4" t="str">
-        <v>4115400234</v>
+        <v>29910200821</v>
       </c>
       <c r="M4" t="str">
-        <v>~441 m (geocode da base)</v>
+        <v>~411 m (geocode da base)</v>
       </c>
       <c r="N4" t="str">
         <v>Abrir no Maps</v>
@@ -949,7 +949,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -957,40 +957,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 74</v>
+        <v>R PROF VAHIA DE ABREU 741</v>
       </c>
       <c r="C5" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D5" t="str">
-        <v>2024-11</v>
+        <v>2024-04</v>
       </c>
       <c r="E5" t="str">
-        <v>247</v>
+        <v>180</v>
       </c>
       <c r="F5" t="str">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="G5" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H5" t="str">
-        <v>R$ 1.200.000</v>
+        <v>R$ 1.320.000</v>
       </c>
       <c r="I5" t="str">
-        <v>4.858</v>
+        <v>7.333</v>
       </c>
       <c r="J5" t="str">
-        <v>1.0648</v>
+        <v>1.1098</v>
       </c>
       <c r="K5" t="str">
-        <v>5.173</v>
+        <v>8.139</v>
       </c>
       <c r="L5" t="str">
-        <v>4123100104</v>
+        <v>29910900597</v>
       </c>
       <c r="M5" t="str">
-        <v>~456 m (geocode da base)</v>
+        <v>~552 m (geocode da base)</v>
       </c>
       <c r="N5" t="str">
         <v>Abrir no Maps</v>
@@ -1013,40 +1013,40 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 77</v>
+        <v>PC CEL FERNANDES DE LIMA 100</v>
       </c>
       <c r="C6" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D6" t="str">
-        <v>2024-03</v>
+        <v>2025-02</v>
       </c>
       <c r="E6" t="str">
-        <v>250</v>
+        <v>154</v>
       </c>
       <c r="F6" t="str">
-        <v>295</v>
+        <v>154</v>
       </c>
       <c r="G6" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H6" t="str">
-        <v>R$ 1.270.000</v>
+        <v>R$ 1.280.000</v>
       </c>
       <c r="I6" t="str">
-        <v>5.080</v>
+        <v>8.312</v>
       </c>
       <c r="J6" t="str">
-        <v>1.1164</v>
+        <v>1.0511</v>
       </c>
       <c r="K6" t="str">
-        <v>5.671</v>
+        <v>8.736</v>
       </c>
       <c r="L6" t="str">
-        <v>4121400089</v>
+        <v>4119300412</v>
       </c>
       <c r="M6" t="str">
-        <v>~458 m (geocode da base)</v>
+        <v>~338 m (geocode da base)</v>
       </c>
       <c r="N6" t="str">
         <v>Abrir no Maps</v>
@@ -1164,40 +1164,40 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>R UBAIRA 60</v>
+        <v>R JURUENA 87</v>
       </c>
       <c r="C2" t="str">
         <v>Moema</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-08</v>
+        <v>2024-11</v>
       </c>
       <c r="E2" t="str">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="F2" t="str">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G2" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H2" t="str">
-        <v>R$ 3.400.000</v>
+        <v>R$ 1.800.000</v>
       </c>
       <c r="I2" t="str">
-        <v>13.600</v>
+        <v>10.000</v>
       </c>
       <c r="J2" t="str">
-        <v>1.0288</v>
+        <v>1.0648</v>
       </c>
       <c r="K2" t="str">
-        <v>13.991</v>
+        <v>10.648</v>
       </c>
       <c r="L2" t="str">
-        <v>4117200224</v>
+        <v>4117200100</v>
       </c>
       <c r="M2" t="str">
-        <v>~282 m (geocode da base)</v>
+        <v>~272 m (geocode da base)</v>
       </c>
       <c r="N2" t="str">
         <v>Abrir no Maps</v>
@@ -1220,40 +1220,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>R JURUENA 87</v>
+        <v>R PARIQUERA-ACU 41</v>
       </c>
       <c r="C3" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D3" t="str">
-        <v>2024-11</v>
+        <v>2026-03</v>
       </c>
       <c r="E3" t="str">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="F3" t="str">
-        <v>303</v>
+        <v>—</v>
       </c>
       <c r="G3" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H3" t="str">
-        <v>R$ 1.800.000</v>
+        <v>R$ 2.500.000</v>
       </c>
       <c r="I3" t="str">
-        <v>10.000</v>
+        <v>12.438</v>
       </c>
       <c r="J3" t="str">
-        <v>1.0648</v>
+        <v>1.0050</v>
       </c>
       <c r="K3" t="str">
-        <v>10.648</v>
+        <v>12.500</v>
       </c>
       <c r="L3" t="str">
-        <v>4117200100</v>
+        <v>4115400234</v>
       </c>
       <c r="M3" t="str">
-        <v>~272 m (geocode da base)</v>
+        <v>~441 m (geocode da base)</v>
       </c>
       <c r="N3" t="str">
         <v>Abrir no Maps</v>
@@ -1268,7 +1268,7 @@
         <v/>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="4">
@@ -1276,40 +1276,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>R PARIQUERA-ACU 41</v>
+        <v>TV SEBASTIAO EMILIO FORLI 58</v>
       </c>
       <c r="C4" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-03</v>
+        <v>2024-05</v>
       </c>
       <c r="E4" t="str">
-        <v>201</v>
+        <v>177</v>
       </c>
       <c r="F4" t="str">
-        <v>—</v>
+        <v>116</v>
       </c>
       <c r="G4" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H4" t="str">
-        <v>R$ 2.500.000</v>
+        <v>R$ 2.900.000</v>
       </c>
       <c r="I4" t="str">
-        <v>12.438</v>
+        <v>16.384</v>
       </c>
       <c r="J4" t="str">
-        <v>1.0050</v>
+        <v>1.1019</v>
       </c>
       <c r="K4" t="str">
-        <v>12.500</v>
+        <v>18.054</v>
       </c>
       <c r="L4" t="str">
-        <v>4115400234</v>
+        <v>29910200821</v>
       </c>
       <c r="M4" t="str">
-        <v>~441 m (geocode da base)</v>
+        <v>~411 m (geocode da base)</v>
       </c>
       <c r="N4" t="str">
         <v>Abrir no Maps</v>
@@ -1324,7 +1324,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -1332,40 +1332,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 74</v>
+        <v>R PROF VAHIA DE ABREU 741</v>
       </c>
       <c r="C5" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D5" t="str">
-        <v>2024-11</v>
+        <v>2024-04</v>
       </c>
       <c r="E5" t="str">
-        <v>247</v>
+        <v>180</v>
       </c>
       <c r="F5" t="str">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="G5" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H5" t="str">
-        <v>R$ 1.200.000</v>
+        <v>R$ 1.320.000</v>
       </c>
       <c r="I5" t="str">
-        <v>4.858</v>
+        <v>7.333</v>
       </c>
       <c r="J5" t="str">
-        <v>1.0648</v>
+        <v>1.1098</v>
       </c>
       <c r="K5" t="str">
-        <v>5.173</v>
+        <v>8.139</v>
       </c>
       <c r="L5" t="str">
-        <v>4123100104</v>
+        <v>29910900597</v>
       </c>
       <c r="M5" t="str">
-        <v>~456 m (geocode da base)</v>
+        <v>~552 m (geocode da base)</v>
       </c>
       <c r="N5" t="str">
         <v>Abrir no Maps</v>
@@ -1388,40 +1388,40 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 77</v>
+        <v>PC CEL FERNANDES DE LIMA 100</v>
       </c>
       <c r="C6" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D6" t="str">
-        <v>2024-03</v>
+        <v>2025-02</v>
       </c>
       <c r="E6" t="str">
-        <v>250</v>
+        <v>154</v>
       </c>
       <c r="F6" t="str">
-        <v>295</v>
+        <v>154</v>
       </c>
       <c r="G6" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H6" t="str">
-        <v>R$ 1.270.000</v>
+        <v>R$ 1.280.000</v>
       </c>
       <c r="I6" t="str">
-        <v>5.080</v>
+        <v>8.312</v>
       </c>
       <c r="J6" t="str">
-        <v>1.1164</v>
+        <v>1.0511</v>
       </c>
       <c r="K6" t="str">
-        <v>5.671</v>
+        <v>8.736</v>
       </c>
       <c r="L6" t="str">
-        <v>4121400089</v>
+        <v>4119300412</v>
       </c>
       <c r="M6" t="str">
-        <v>~458 m (geocode da base)</v>
+        <v>~338 m (geocode da base)</v>
       </c>
       <c r="N6" t="str">
         <v>Abrir no Maps</v>
@@ -1444,40 +1444,40 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>R IRAUNA 669</v>
+        <v>R ILAMONIA 203</v>
       </c>
       <c r="C7" t="str">
         <v>Moema</v>
       </c>
       <c r="D7" t="str">
-        <v>2024-06</v>
+        <v>2025-08</v>
       </c>
       <c r="E7" t="str">
-        <v>231</v>
+        <v>184</v>
       </c>
       <c r="F7" t="str">
-        <v>312</v>
+        <v>170</v>
       </c>
       <c r="G7" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H7" t="str">
-        <v>R$ 1.400.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I7" t="str">
-        <v>6.061</v>
+        <v>8.152</v>
       </c>
       <c r="J7" t="str">
-        <v>1.0944</v>
+        <v>1.0288</v>
       </c>
       <c r="K7" t="str">
-        <v>6.633</v>
+        <v>8.387</v>
       </c>
       <c r="L7" t="str">
-        <v>4121700041</v>
+        <v>4119600319</v>
       </c>
       <c r="M7" t="str">
-        <v>~617 m (geocode da base)</v>
+        <v>~612 m (geocode da base)</v>
       </c>
       <c r="N7" t="str">
         <v>Abrir no Maps</v>
@@ -1500,40 +1500,40 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>TV SEBASTIAO EMILIO FORLI 58</v>
+        <v>R UBAIRA 60</v>
       </c>
       <c r="C8" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D8" t="str">
-        <v>2024-05</v>
+        <v>2025-08</v>
       </c>
       <c r="E8" t="str">
-        <v>177</v>
+        <v>250</v>
       </c>
       <c r="F8" t="str">
-        <v>116</v>
+        <v>305</v>
       </c>
       <c r="G8" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H8" t="str">
-        <v>R$ 2.900.000</v>
+        <v>R$ 3.400.000</v>
       </c>
       <c r="I8" t="str">
-        <v>16.384</v>
+        <v>13.600</v>
       </c>
       <c r="J8" t="str">
-        <v>1.1019</v>
+        <v>1.0288</v>
       </c>
       <c r="K8" t="str">
-        <v>18.054</v>
+        <v>13.991</v>
       </c>
       <c r="L8" t="str">
-        <v>29910200821</v>
+        <v>4117200224</v>
       </c>
       <c r="M8" t="str">
-        <v>~411 m (geocode da base)</v>
+        <v>~282 m (geocode da base)</v>
       </c>
       <c r="N8" t="str">
         <v>Abrir no Maps</v>
@@ -1556,40 +1556,40 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>R IRAUNA 655</v>
+        <v>R ELIAS FAUSTO 34</v>
       </c>
       <c r="C9" t="str">
         <v>Moema</v>
       </c>
       <c r="D9" t="str">
-        <v>2024-02</v>
+        <v>2024-05</v>
       </c>
       <c r="E9" t="str">
-        <v>248</v>
+        <v>164</v>
       </c>
       <c r="F9" t="str">
-        <v>312</v>
+        <v>145</v>
       </c>
       <c r="G9" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H9" t="str">
-        <v>R$ 2.350.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I9" t="str">
-        <v>9.476</v>
+        <v>11.738</v>
       </c>
       <c r="J9" t="str">
-        <v>1.1221</v>
+        <v>1.1019</v>
       </c>
       <c r="K9" t="str">
-        <v>10.633</v>
+        <v>12.934</v>
       </c>
       <c r="L9" t="str">
-        <v>4121700120</v>
+        <v>4115500239</v>
       </c>
       <c r="M9" t="str">
-        <v>~604 m (geocode da base)</v>
+        <v>~549 m (geocode da base)</v>
       </c>
       <c r="N9" t="str">
         <v>Abrir no Maps</v>
@@ -1612,40 +1612,40 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>PC CEL FERNANDES DE LIMA 100</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 476</v>
       </c>
       <c r="C10" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-02</v>
+        <v>2024-07</v>
       </c>
       <c r="E10" t="str">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="F10" t="str">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="G10" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H10" t="str">
-        <v>R$ 1.280.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I10" t="str">
-        <v>8.312</v>
+        <v>7.895</v>
       </c>
       <c r="J10" t="str">
-        <v>1.0511</v>
+        <v>1.0879</v>
       </c>
       <c r="K10" t="str">
-        <v>8.736</v>
+        <v>8.589</v>
       </c>
       <c r="L10" t="str">
-        <v>4119300412</v>
+        <v>4127700270</v>
       </c>
       <c r="M10" t="str">
-        <v>~338 m (geocode da base)</v>
+        <v>~789 m (geocode da base)</v>
       </c>
       <c r="N10" t="str">
         <v>Abrir no Maps</v>
@@ -1668,40 +1668,40 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>R PROF VAHIA DE ABREU 741</v>
+        <v>R ELIAS FAUSTO 40</v>
       </c>
       <c r="C11" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D11" t="str">
-        <v>2024-04</v>
+        <v>2024-05</v>
       </c>
       <c r="E11" t="str">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="F11" t="str">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="G11" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H11" t="str">
-        <v>R$ 1.320.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I11" t="str">
-        <v>7.333</v>
+        <v>12.031</v>
       </c>
       <c r="J11" t="str">
-        <v>1.1098</v>
+        <v>1.1019</v>
       </c>
       <c r="K11" t="str">
-        <v>8.139</v>
+        <v>13.258</v>
       </c>
       <c r="L11" t="str">
-        <v>29910900597</v>
+        <v>4115500247</v>
       </c>
       <c r="M11" t="str">
-        <v>~552 m (geocode da base)</v>
+        <v>~549 m (geocode da base)</v>
       </c>
       <c r="N11" t="str">
         <v>Abrir no Maps</v>
@@ -1824,40 +1824,40 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>R UBAIRA 60</v>
+        <v>R JURUENA 87</v>
       </c>
       <c r="C2" t="str">
         <v>Moema</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-08</v>
+        <v>2024-11</v>
       </c>
       <c r="E2" t="str">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="F2" t="str">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G2" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H2" t="str">
-        <v>R$ 3.400.000</v>
+        <v>R$ 1.800.000</v>
       </c>
       <c r="I2" t="str">
-        <v>13.600</v>
+        <v>10.000</v>
       </c>
       <c r="J2" t="str">
-        <v>1.0288</v>
+        <v>1.0648</v>
       </c>
       <c r="K2" t="str">
-        <v>13.991</v>
+        <v>10.648</v>
       </c>
       <c r="L2" t="str">
-        <v>4117200224</v>
+        <v>4117200100</v>
       </c>
       <c r="M2" t="str">
-        <v>~282 m (geocode da base)</v>
+        <v>~272 m (geocode da base)</v>
       </c>
       <c r="N2" t="str">
         <v>Abrir no Maps</v>
@@ -1880,40 +1880,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>R JURUENA 87</v>
+        <v>R PARIQUERA-ACU 41</v>
       </c>
       <c r="C3" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D3" t="str">
-        <v>2024-11</v>
+        <v>2026-03</v>
       </c>
       <c r="E3" t="str">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="F3" t="str">
-        <v>303</v>
+        <v>—</v>
       </c>
       <c r="G3" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H3" t="str">
-        <v>R$ 1.800.000</v>
+        <v>R$ 2.500.000</v>
       </c>
       <c r="I3" t="str">
-        <v>10.000</v>
+        <v>12.438</v>
       </c>
       <c r="J3" t="str">
-        <v>1.0648</v>
+        <v>1.0050</v>
       </c>
       <c r="K3" t="str">
-        <v>10.648</v>
+        <v>12.500</v>
       </c>
       <c r="L3" t="str">
-        <v>4117200100</v>
+        <v>4115400234</v>
       </c>
       <c r="M3" t="str">
-        <v>~272 m (geocode da base)</v>
+        <v>~441 m (geocode da base)</v>
       </c>
       <c r="N3" t="str">
         <v>Abrir no Maps</v>
@@ -1928,7 +1928,7 @@
         <v/>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="4">
@@ -1936,40 +1936,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>R PARIQUERA-ACU 41</v>
+        <v>TV SEBASTIAO EMILIO FORLI 58</v>
       </c>
       <c r="C4" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-03</v>
+        <v>2024-05</v>
       </c>
       <c r="E4" t="str">
-        <v>201</v>
+        <v>177</v>
       </c>
       <c r="F4" t="str">
-        <v>—</v>
+        <v>116</v>
       </c>
       <c r="G4" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H4" t="str">
-        <v>R$ 2.500.000</v>
+        <v>R$ 2.900.000</v>
       </c>
       <c r="I4" t="str">
-        <v>12.438</v>
+        <v>16.384</v>
       </c>
       <c r="J4" t="str">
-        <v>1.0050</v>
+        <v>1.1019</v>
       </c>
       <c r="K4" t="str">
-        <v>12.500</v>
+        <v>18.054</v>
       </c>
       <c r="L4" t="str">
-        <v>4115400234</v>
+        <v>29910200821</v>
       </c>
       <c r="M4" t="str">
-        <v>~441 m (geocode da base)</v>
+        <v>~411 m (geocode da base)</v>
       </c>
       <c r="N4" t="str">
         <v>Abrir no Maps</v>
@@ -1984,7 +1984,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -1992,40 +1992,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 74</v>
+        <v>R PROF VAHIA DE ABREU 741</v>
       </c>
       <c r="C5" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D5" t="str">
-        <v>2024-11</v>
+        <v>2024-04</v>
       </c>
       <c r="E5" t="str">
-        <v>247</v>
+        <v>180</v>
       </c>
       <c r="F5" t="str">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="G5" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H5" t="str">
-        <v>R$ 1.200.000</v>
+        <v>R$ 1.320.000</v>
       </c>
       <c r="I5" t="str">
-        <v>4.858</v>
+        <v>7.333</v>
       </c>
       <c r="J5" t="str">
-        <v>1.0648</v>
+        <v>1.1098</v>
       </c>
       <c r="K5" t="str">
-        <v>5.173</v>
+        <v>8.139</v>
       </c>
       <c r="L5" t="str">
-        <v>4123100104</v>
+        <v>29910900597</v>
       </c>
       <c r="M5" t="str">
-        <v>~456 m (geocode da base)</v>
+        <v>~552 m (geocode da base)</v>
       </c>
       <c r="N5" t="str">
         <v>Abrir no Maps</v>
@@ -2048,40 +2048,40 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 77</v>
+        <v>PC CEL FERNANDES DE LIMA 100</v>
       </c>
       <c r="C6" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D6" t="str">
-        <v>2024-03</v>
+        <v>2025-02</v>
       </c>
       <c r="E6" t="str">
-        <v>250</v>
+        <v>154</v>
       </c>
       <c r="F6" t="str">
-        <v>295</v>
+        <v>154</v>
       </c>
       <c r="G6" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H6" t="str">
-        <v>R$ 1.270.000</v>
+        <v>R$ 1.280.000</v>
       </c>
       <c r="I6" t="str">
-        <v>5.080</v>
+        <v>8.312</v>
       </c>
       <c r="J6" t="str">
-        <v>1.1164</v>
+        <v>1.0511</v>
       </c>
       <c r="K6" t="str">
-        <v>5.671</v>
+        <v>8.736</v>
       </c>
       <c r="L6" t="str">
-        <v>4121400089</v>
+        <v>4119300412</v>
       </c>
       <c r="M6" t="str">
-        <v>~458 m (geocode da base)</v>
+        <v>~338 m (geocode da base)</v>
       </c>
       <c r="N6" t="str">
         <v>Abrir no Maps</v>
@@ -2104,40 +2104,40 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>R IRAUNA 669</v>
+        <v>R ILAMONIA 203</v>
       </c>
       <c r="C7" t="str">
         <v>Moema</v>
       </c>
       <c r="D7" t="str">
-        <v>2024-06</v>
+        <v>2025-08</v>
       </c>
       <c r="E7" t="str">
-        <v>231</v>
+        <v>184</v>
       </c>
       <c r="F7" t="str">
-        <v>312</v>
+        <v>170</v>
       </c>
       <c r="G7" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H7" t="str">
-        <v>R$ 1.400.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I7" t="str">
-        <v>6.061</v>
+        <v>8.152</v>
       </c>
       <c r="J7" t="str">
-        <v>1.0944</v>
+        <v>1.0288</v>
       </c>
       <c r="K7" t="str">
-        <v>6.633</v>
+        <v>8.387</v>
       </c>
       <c r="L7" t="str">
-        <v>4121700041</v>
+        <v>4119600319</v>
       </c>
       <c r="M7" t="str">
-        <v>~617 m (geocode da base)</v>
+        <v>~612 m (geocode da base)</v>
       </c>
       <c r="N7" t="str">
         <v>Abrir no Maps</v>
@@ -2160,40 +2160,40 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>TV SEBASTIAO EMILIO FORLI 58</v>
+        <v>R UBAIRA 60</v>
       </c>
       <c r="C8" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D8" t="str">
-        <v>2024-05</v>
+        <v>2025-08</v>
       </c>
       <c r="E8" t="str">
-        <v>177</v>
+        <v>250</v>
       </c>
       <c r="F8" t="str">
-        <v>116</v>
+        <v>305</v>
       </c>
       <c r="G8" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H8" t="str">
-        <v>R$ 2.900.000</v>
+        <v>R$ 3.400.000</v>
       </c>
       <c r="I8" t="str">
-        <v>16.384</v>
+        <v>13.600</v>
       </c>
       <c r="J8" t="str">
-        <v>1.1019</v>
+        <v>1.0288</v>
       </c>
       <c r="K8" t="str">
-        <v>18.054</v>
+        <v>13.991</v>
       </c>
       <c r="L8" t="str">
-        <v>29910200821</v>
+        <v>4117200224</v>
       </c>
       <c r="M8" t="str">
-        <v>~411 m (geocode da base)</v>
+        <v>~282 m (geocode da base)</v>
       </c>
       <c r="N8" t="str">
         <v>Abrir no Maps</v>
@@ -2216,40 +2216,40 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>R IRAUNA 655</v>
+        <v>R ELIAS FAUSTO 34</v>
       </c>
       <c r="C9" t="str">
         <v>Moema</v>
       </c>
       <c r="D9" t="str">
-        <v>2024-02</v>
+        <v>2024-05</v>
       </c>
       <c r="E9" t="str">
-        <v>248</v>
+        <v>164</v>
       </c>
       <c r="F9" t="str">
-        <v>312</v>
+        <v>145</v>
       </c>
       <c r="G9" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H9" t="str">
-        <v>R$ 2.350.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I9" t="str">
-        <v>9.476</v>
+        <v>11.738</v>
       </c>
       <c r="J9" t="str">
-        <v>1.1221</v>
+        <v>1.1019</v>
       </c>
       <c r="K9" t="str">
-        <v>10.633</v>
+        <v>12.934</v>
       </c>
       <c r="L9" t="str">
-        <v>4121700120</v>
+        <v>4115500239</v>
       </c>
       <c r="M9" t="str">
-        <v>~604 m (geocode da base)</v>
+        <v>~549 m (geocode da base)</v>
       </c>
       <c r="N9" t="str">
         <v>Abrir no Maps</v>
@@ -2272,40 +2272,40 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>PC CEL FERNANDES DE LIMA 100</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 476</v>
       </c>
       <c r="C10" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-02</v>
+        <v>2024-07</v>
       </c>
       <c r="E10" t="str">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="F10" t="str">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="G10" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H10" t="str">
-        <v>R$ 1.280.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I10" t="str">
-        <v>8.312</v>
+        <v>7.895</v>
       </c>
       <c r="J10" t="str">
-        <v>1.0511</v>
+        <v>1.0879</v>
       </c>
       <c r="K10" t="str">
-        <v>8.736</v>
+        <v>8.589</v>
       </c>
       <c r="L10" t="str">
-        <v>4119300412</v>
+        <v>4127700270</v>
       </c>
       <c r="M10" t="str">
-        <v>~338 m (geocode da base)</v>
+        <v>~789 m (geocode da base)</v>
       </c>
       <c r="N10" t="str">
         <v>Abrir no Maps</v>
@@ -2328,40 +2328,40 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>R PROF VAHIA DE ABREU 741</v>
+        <v>R ELIAS FAUSTO 40</v>
       </c>
       <c r="C11" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D11" t="str">
-        <v>2024-04</v>
+        <v>2024-05</v>
       </c>
       <c r="E11" t="str">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="F11" t="str">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="G11" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H11" t="str">
-        <v>R$ 1.320.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I11" t="str">
-        <v>7.333</v>
+        <v>12.031</v>
       </c>
       <c r="J11" t="str">
-        <v>1.1098</v>
+        <v>1.1019</v>
       </c>
       <c r="K11" t="str">
-        <v>8.139</v>
+        <v>13.258</v>
       </c>
       <c r="L11" t="str">
-        <v>29910900597</v>
+        <v>4115500247</v>
       </c>
       <c r="M11" t="str">
-        <v>~552 m (geocode da base)</v>
+        <v>~549 m (geocode da base)</v>
       </c>
       <c r="N11" t="str">
         <v>Abrir no Maps</v>
@@ -2440,40 +2440,40 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>R MARIA NOSCHESE 315</v>
+        <v>R ARAGUARI 239</v>
       </c>
       <c r="C13" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D13" t="str">
-        <v>2024-03</v>
+        <v>2025-10</v>
       </c>
       <c r="E13" t="str">
-        <v>230</v>
+        <v>190</v>
       </c>
       <c r="F13" t="str">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G13" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H13" t="str">
-        <v>R$ 1.400.000</v>
+        <v>R$ 1.900.000</v>
       </c>
       <c r="I13" t="str">
-        <v>6.087</v>
+        <v>10.000</v>
       </c>
       <c r="J13" t="str">
-        <v>1.1164</v>
+        <v>1.0190</v>
       </c>
       <c r="K13" t="str">
-        <v>6.796</v>
+        <v>10.190</v>
       </c>
       <c r="L13" t="str">
-        <v>4127700327</v>
+        <v>4108000171</v>
       </c>
       <c r="M13" t="str">
-        <v>~800 m (geocode da base)</v>
+        <v>~816 m (geocode da base)</v>
       </c>
       <c r="N13" t="str">
         <v>Abrir no Maps</v>
@@ -2496,40 +2496,40 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>R ILAMONIA 203</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 74</v>
       </c>
       <c r="C14" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-08</v>
+        <v>2024-11</v>
       </c>
       <c r="E14" t="str">
-        <v>184</v>
+        <v>247</v>
       </c>
       <c r="F14" t="str">
-        <v>170</v>
+        <v>280</v>
       </c>
       <c r="G14" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H14" t="str">
-        <v>R$ 1.500.000</v>
+        <v>R$ 1.200.000</v>
       </c>
       <c r="I14" t="str">
-        <v>8.152</v>
+        <v>4.858</v>
       </c>
       <c r="J14" t="str">
-        <v>1.0288</v>
+        <v>1.0648</v>
       </c>
       <c r="K14" t="str">
-        <v>8.387</v>
+        <v>5.173</v>
       </c>
       <c r="L14" t="str">
-        <v>4119600319</v>
+        <v>4123100104</v>
       </c>
       <c r="M14" t="str">
-        <v>~612 m (geocode da base)</v>
+        <v>~456 m (geocode da base)</v>
       </c>
       <c r="N14" t="str">
         <v>Abrir no Maps</v>
@@ -2552,40 +2552,40 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>AL DOS ARAPANES 1671</v>
+        <v>R IRAUNA 669</v>
       </c>
       <c r="C15" t="str">
         <v>Moema</v>
       </c>
       <c r="D15" t="str">
-        <v>2024-10</v>
+        <v>2024-06</v>
       </c>
       <c r="E15" t="str">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="F15" t="str">
-        <v>—</v>
+        <v>312</v>
       </c>
       <c r="G15" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H15" t="str">
-        <v>R$ 2.800.000</v>
+        <v>R$ 1.400.000</v>
       </c>
       <c r="I15" t="str">
-        <v>12.670</v>
+        <v>6.061</v>
       </c>
       <c r="J15" t="str">
-        <v>1.0697</v>
+        <v>1.0944</v>
       </c>
       <c r="K15" t="str">
-        <v>13.552</v>
+        <v>6.633</v>
       </c>
       <c r="L15" t="str">
-        <v>4122000041</v>
+        <v>4121700041</v>
       </c>
       <c r="M15" t="str">
-        <v>~901 m (geocode da base)</v>
+        <v>~617 m (geocode da base)</v>
       </c>
       <c r="N15" t="str">
         <v>Abrir no Maps</v>
@@ -2600,7 +2600,7 @@
         <v/>
       </c>
       <c r="R15" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -2608,40 +2608,40 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>R IRAUNA 550</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 77</v>
       </c>
       <c r="C16" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D16" t="str">
-        <v>2024-04</v>
+        <v>2024-03</v>
       </c>
       <c r="E16" t="str">
-        <v>279</v>
+        <v>250</v>
       </c>
       <c r="F16" t="str">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="G16" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H16" t="str">
-        <v>R$ 1.900.000</v>
+        <v>R$ 1.270.000</v>
       </c>
       <c r="I16" t="str">
-        <v>6.810</v>
+        <v>5.080</v>
       </c>
       <c r="J16" t="str">
-        <v>1.1098</v>
+        <v>1.1164</v>
       </c>
       <c r="K16" t="str">
-        <v>7.558</v>
+        <v>5.671</v>
       </c>
       <c r="L16" t="str">
-        <v>4121500180</v>
+        <v>4121400089</v>
       </c>
       <c r="M16" t="str">
-        <v>~508 m (geocode da base)</v>
+        <v>~458 m (geocode da base)</v>
       </c>
       <c r="N16" t="str">
         <v>Abrir no Maps</v>
@@ -2664,40 +2664,40 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>R ELIAS FAUSTO 34</v>
+        <v>R EMB RIBEIRO COUTO 286</v>
       </c>
       <c r="C17" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D17" t="str">
-        <v>2024-05</v>
+        <v>2025-10</v>
       </c>
       <c r="E17" t="str">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F17" t="str">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="G17" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H17" t="str">
-        <v>R$ 1.925.000</v>
+        <v>R$ 1.700.000</v>
       </c>
       <c r="I17" t="str">
-        <v>11.738</v>
+        <v>10.303</v>
       </c>
       <c r="J17" t="str">
-        <v>1.1019</v>
+        <v>1.0190</v>
       </c>
       <c r="K17" t="str">
-        <v>12.934</v>
+        <v>10.499</v>
       </c>
       <c r="L17" t="str">
-        <v>4115500239</v>
+        <v>4119700437</v>
       </c>
       <c r="M17" t="str">
-        <v>~549 m (geocode da base)</v>
+        <v>~679 m (geocode da base)</v>
       </c>
       <c r="N17" t="str">
         <v>Abrir no Maps</v>
@@ -2720,40 +2720,40 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>R CEL DAVIO ESPIRIDIAO 10</v>
+        <v>R GAIVOTA 1622</v>
       </c>
       <c r="C18" t="str">
         <v>Moema</v>
       </c>
       <c r="D18" t="str">
-        <v>2026-01</v>
+        <v>2025-03</v>
       </c>
       <c r="E18" t="str">
-        <v>275</v>
+        <v>150</v>
       </c>
       <c r="F18" t="str">
-        <v>—</v>
+        <v>187</v>
       </c>
       <c r="G18" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H18" t="str">
-        <v>R$ 3.750.000</v>
+        <v>R$ 1.650.000</v>
       </c>
       <c r="I18" t="str">
-        <v>13.636</v>
+        <v>11.000</v>
       </c>
       <c r="J18" t="str">
-        <v>1.0117</v>
+        <v>1.0488</v>
       </c>
       <c r="K18" t="str">
-        <v>13.796</v>
+        <v>11.537</v>
       </c>
       <c r="L18" t="str">
-        <v>4115700408</v>
+        <v>4119600270</v>
       </c>
       <c r="M18" t="str">
-        <v>~578 m (geocode da base)</v>
+        <v>~624 m (geocode da base)</v>
       </c>
       <c r="N18" t="str">
         <v>Abrir no Maps</v>
@@ -2768,7 +2768,7 @@
         <v/>
       </c>
       <c r="R18" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -2776,40 +2776,40 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>R ELIAS FAUSTO 40</v>
+        <v>R EMB RIBEIRO COUTO 302</v>
       </c>
       <c r="C19" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D19" t="str">
-        <v>2024-05</v>
+        <v>2025-08</v>
       </c>
       <c r="E19" t="str">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F19" t="str">
-        <v>139</v>
+        <v>264</v>
       </c>
       <c r="G19" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H19" t="str">
-        <v>R$ 1.925.000</v>
+        <v>R$ 1.540.000</v>
       </c>
       <c r="I19" t="str">
-        <v>12.031</v>
+        <v>9.935</v>
       </c>
       <c r="J19" t="str">
-        <v>1.1019</v>
+        <v>1.0288</v>
       </c>
       <c r="K19" t="str">
-        <v>13.258</v>
+        <v>10.221</v>
       </c>
       <c r="L19" t="str">
-        <v>4115500247</v>
+        <v>4119700410</v>
       </c>
       <c r="M19" t="str">
-        <v>~549 m (geocode da base)</v>
+        <v>~694 m (geocode da base)</v>
       </c>
       <c r="N19" t="str">
         <v>Abrir no Maps</v>
@@ -2832,40 +2832,40 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 476</v>
+        <v>R IRAUNA 615</v>
       </c>
       <c r="C20" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D20" t="str">
-        <v>2024-07</v>
+        <v>2024-03</v>
       </c>
       <c r="E20" t="str">
-        <v>190</v>
+        <v>140</v>
       </c>
       <c r="F20" t="str">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="G20" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H20" t="str">
-        <v>R$ 1.500.000</v>
+        <v>R$ 1.440.000</v>
       </c>
       <c r="I20" t="str">
-        <v>7.895</v>
+        <v>10.286</v>
       </c>
       <c r="J20" t="str">
-        <v>1.0879</v>
+        <v>1.1164</v>
       </c>
       <c r="K20" t="str">
-        <v>8.589</v>
+        <v>11.483</v>
       </c>
       <c r="L20" t="str">
-        <v>4127700270</v>
+        <v>4121700211</v>
       </c>
       <c r="M20" t="str">
-        <v>~789 m (geocode da base)</v>
+        <v>~569 m (geocode da base)</v>
       </c>
       <c r="N20" t="str">
         <v>Abrir no Maps</v>
@@ -2888,40 +2888,40 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>AL DOS ARAPANES 1855</v>
+        <v>R IRAUNA 655</v>
       </c>
       <c r="C21" t="str">
         <v>Moema</v>
       </c>
       <c r="D21" t="str">
-        <v>2026-04</v>
+        <v>2024-02</v>
       </c>
       <c r="E21" t="str">
-        <v>212</v>
+        <v>248</v>
       </c>
       <c r="F21" t="str">
-        <v>—</v>
+        <v>312</v>
       </c>
       <c r="G21" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H21" t="str">
-        <v>R$ 1.925.000</v>
+        <v>R$ 2.350.000</v>
       </c>
       <c r="I21" t="str">
-        <v>9.080</v>
+        <v>9.476</v>
       </c>
       <c r="J21" t="str">
-        <v>1.0030</v>
+        <v>1.1221</v>
       </c>
       <c r="K21" t="str">
-        <v>9.108</v>
+        <v>10.633</v>
       </c>
       <c r="L21" t="str">
-        <v>4127900083</v>
+        <v>4121700120</v>
       </c>
       <c r="M21" t="str">
-        <v>~956 m (geocode da base)</v>
+        <v>~604 m (geocode da base)</v>
       </c>
       <c r="N21" t="str">
         <v>Abrir no Maps</v>
@@ -2936,7 +2936,7 @@
         <v/>
       </c>
       <c r="R21" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3054,40 +3054,40 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>R UBAIRA 60</v>
+        <v>R JURUENA 87</v>
       </c>
       <c r="C2" t="str">
         <v>Moema</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-08</v>
+        <v>2024-11</v>
       </c>
       <c r="E2" t="str">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="F2" t="str">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G2" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H2" t="str">
-        <v>R$ 3.400.000</v>
+        <v>R$ 1.800.000</v>
       </c>
       <c r="I2" t="str">
-        <v>13.600</v>
+        <v>10.000</v>
       </c>
       <c r="J2" t="str">
-        <v>1.0288</v>
+        <v>1.0648</v>
       </c>
       <c r="K2" t="str">
-        <v>13.991</v>
+        <v>10.648</v>
       </c>
       <c r="L2" t="str">
-        <v>4117200224</v>
+        <v>4117200100</v>
       </c>
       <c r="M2" t="str">
-        <v>~282 m (geocode da base)</v>
+        <v>~272 m (geocode da base)</v>
       </c>
       <c r="N2" t="str">
         <v>Abrir no Maps</v>
@@ -3110,40 +3110,40 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>R JURUENA 87</v>
+        <v>R PARIQUERA-ACU 41</v>
       </c>
       <c r="C3" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D3" t="str">
-        <v>2024-11</v>
+        <v>2026-03</v>
       </c>
       <c r="E3" t="str">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="F3" t="str">
-        <v>303</v>
+        <v>—</v>
       </c>
       <c r="G3" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H3" t="str">
-        <v>R$ 1.800.000</v>
+        <v>R$ 2.500.000</v>
       </c>
       <c r="I3" t="str">
-        <v>10.000</v>
+        <v>12.438</v>
       </c>
       <c r="J3" t="str">
-        <v>1.0648</v>
+        <v>1.0050</v>
       </c>
       <c r="K3" t="str">
-        <v>10.648</v>
+        <v>12.500</v>
       </c>
       <c r="L3" t="str">
-        <v>4117200100</v>
+        <v>4115400234</v>
       </c>
       <c r="M3" t="str">
-        <v>~272 m (geocode da base)</v>
+        <v>~441 m (geocode da base)</v>
       </c>
       <c r="N3" t="str">
         <v>Abrir no Maps</v>
@@ -3158,7 +3158,7 @@
         <v/>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="4">
@@ -3166,40 +3166,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>R PARIQUERA-ACU 41</v>
+        <v>TV SEBASTIAO EMILIO FORLI 58</v>
       </c>
       <c r="C4" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-03</v>
+        <v>2024-05</v>
       </c>
       <c r="E4" t="str">
-        <v>201</v>
+        <v>177</v>
       </c>
       <c r="F4" t="str">
-        <v>—</v>
+        <v>116</v>
       </c>
       <c r="G4" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H4" t="str">
-        <v>R$ 2.500.000</v>
+        <v>R$ 2.900.000</v>
       </c>
       <c r="I4" t="str">
-        <v>12.438</v>
+        <v>16.384</v>
       </c>
       <c r="J4" t="str">
-        <v>1.0050</v>
+        <v>1.1019</v>
       </c>
       <c r="K4" t="str">
-        <v>12.500</v>
+        <v>18.054</v>
       </c>
       <c r="L4" t="str">
-        <v>4115400234</v>
+        <v>29910200821</v>
       </c>
       <c r="M4" t="str">
-        <v>~441 m (geocode da base)</v>
+        <v>~411 m (geocode da base)</v>
       </c>
       <c r="N4" t="str">
         <v>Abrir no Maps</v>
@@ -3214,7 +3214,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -3222,40 +3222,40 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 74</v>
+        <v>R PROF VAHIA DE ABREU 741</v>
       </c>
       <c r="C5" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D5" t="str">
-        <v>2024-11</v>
+        <v>2024-04</v>
       </c>
       <c r="E5" t="str">
-        <v>247</v>
+        <v>180</v>
       </c>
       <c r="F5" t="str">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="G5" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H5" t="str">
-        <v>R$ 1.200.000</v>
+        <v>R$ 1.320.000</v>
       </c>
       <c r="I5" t="str">
-        <v>4.858</v>
+        <v>7.333</v>
       </c>
       <c r="J5" t="str">
-        <v>1.0648</v>
+        <v>1.1098</v>
       </c>
       <c r="K5" t="str">
-        <v>5.173</v>
+        <v>8.139</v>
       </c>
       <c r="L5" t="str">
-        <v>4123100104</v>
+        <v>29910900597</v>
       </c>
       <c r="M5" t="str">
-        <v>~456 m (geocode da base)</v>
+        <v>~552 m (geocode da base)</v>
       </c>
       <c r="N5" t="str">
         <v>Abrir no Maps</v>
@@ -3278,40 +3278,40 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 77</v>
+        <v>PC CEL FERNANDES DE LIMA 100</v>
       </c>
       <c r="C6" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D6" t="str">
-        <v>2024-03</v>
+        <v>2025-02</v>
       </c>
       <c r="E6" t="str">
-        <v>250</v>
+        <v>154</v>
       </c>
       <c r="F6" t="str">
-        <v>295</v>
+        <v>154</v>
       </c>
       <c r="G6" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H6" t="str">
-        <v>R$ 1.270.000</v>
+        <v>R$ 1.280.000</v>
       </c>
       <c r="I6" t="str">
-        <v>5.080</v>
+        <v>8.312</v>
       </c>
       <c r="J6" t="str">
-        <v>1.1164</v>
+        <v>1.0511</v>
       </c>
       <c r="K6" t="str">
-        <v>5.671</v>
+        <v>8.736</v>
       </c>
       <c r="L6" t="str">
-        <v>4121400089</v>
+        <v>4119300412</v>
       </c>
       <c r="M6" t="str">
-        <v>~458 m (geocode da base)</v>
+        <v>~338 m (geocode da base)</v>
       </c>
       <c r="N6" t="str">
         <v>Abrir no Maps</v>
@@ -3334,40 +3334,40 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>R IRAUNA 669</v>
+        <v>R ILAMONIA 203</v>
       </c>
       <c r="C7" t="str">
         <v>Moema</v>
       </c>
       <c r="D7" t="str">
-        <v>2024-06</v>
+        <v>2025-08</v>
       </c>
       <c r="E7" t="str">
-        <v>231</v>
+        <v>184</v>
       </c>
       <c r="F7" t="str">
-        <v>312</v>
+        <v>170</v>
       </c>
       <c r="G7" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H7" t="str">
-        <v>R$ 1.400.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I7" t="str">
-        <v>6.061</v>
+        <v>8.152</v>
       </c>
       <c r="J7" t="str">
-        <v>1.0944</v>
+        <v>1.0288</v>
       </c>
       <c r="K7" t="str">
-        <v>6.633</v>
+        <v>8.387</v>
       </c>
       <c r="L7" t="str">
-        <v>4121700041</v>
+        <v>4119600319</v>
       </c>
       <c r="M7" t="str">
-        <v>~617 m (geocode da base)</v>
+        <v>~612 m (geocode da base)</v>
       </c>
       <c r="N7" t="str">
         <v>Abrir no Maps</v>
@@ -3390,40 +3390,40 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>TV SEBASTIAO EMILIO FORLI 58</v>
+        <v>R UBAIRA 60</v>
       </c>
       <c r="C8" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D8" t="str">
-        <v>2024-05</v>
+        <v>2025-08</v>
       </c>
       <c r="E8" t="str">
-        <v>177</v>
+        <v>250</v>
       </c>
       <c r="F8" t="str">
-        <v>116</v>
+        <v>305</v>
       </c>
       <c r="G8" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H8" t="str">
-        <v>R$ 2.900.000</v>
+        <v>R$ 3.400.000</v>
       </c>
       <c r="I8" t="str">
-        <v>16.384</v>
+        <v>13.600</v>
       </c>
       <c r="J8" t="str">
-        <v>1.1019</v>
+        <v>1.0288</v>
       </c>
       <c r="K8" t="str">
-        <v>18.054</v>
+        <v>13.991</v>
       </c>
       <c r="L8" t="str">
-        <v>29910200821</v>
+        <v>4117200224</v>
       </c>
       <c r="M8" t="str">
-        <v>~411 m (geocode da base)</v>
+        <v>~282 m (geocode da base)</v>
       </c>
       <c r="N8" t="str">
         <v>Abrir no Maps</v>
@@ -3446,40 +3446,40 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>R IRAUNA 655</v>
+        <v>R ELIAS FAUSTO 34</v>
       </c>
       <c r="C9" t="str">
         <v>Moema</v>
       </c>
       <c r="D9" t="str">
-        <v>2024-02</v>
+        <v>2024-05</v>
       </c>
       <c r="E9" t="str">
-        <v>248</v>
+        <v>164</v>
       </c>
       <c r="F9" t="str">
-        <v>312</v>
+        <v>145</v>
       </c>
       <c r="G9" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H9" t="str">
-        <v>R$ 2.350.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I9" t="str">
-        <v>9.476</v>
+        <v>11.738</v>
       </c>
       <c r="J9" t="str">
-        <v>1.1221</v>
+        <v>1.1019</v>
       </c>
       <c r="K9" t="str">
-        <v>10.633</v>
+        <v>12.934</v>
       </c>
       <c r="L9" t="str">
-        <v>4121700120</v>
+        <v>4115500239</v>
       </c>
       <c r="M9" t="str">
-        <v>~604 m (geocode da base)</v>
+        <v>~549 m (geocode da base)</v>
       </c>
       <c r="N9" t="str">
         <v>Abrir no Maps</v>
@@ -3502,40 +3502,40 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>PC CEL FERNANDES DE LIMA 100</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 476</v>
       </c>
       <c r="C10" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-02</v>
+        <v>2024-07</v>
       </c>
       <c r="E10" t="str">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="F10" t="str">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="G10" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H10" t="str">
-        <v>R$ 1.280.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I10" t="str">
-        <v>8.312</v>
+        <v>7.895</v>
       </c>
       <c r="J10" t="str">
-        <v>1.0511</v>
+        <v>1.0879</v>
       </c>
       <c r="K10" t="str">
-        <v>8.736</v>
+        <v>8.589</v>
       </c>
       <c r="L10" t="str">
-        <v>4119300412</v>
+        <v>4127700270</v>
       </c>
       <c r="M10" t="str">
-        <v>~338 m (geocode da base)</v>
+        <v>~789 m (geocode da base)</v>
       </c>
       <c r="N10" t="str">
         <v>Abrir no Maps</v>
@@ -3558,40 +3558,40 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>R PROF VAHIA DE ABREU 741</v>
+        <v>R ELIAS FAUSTO 40</v>
       </c>
       <c r="C11" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D11" t="str">
-        <v>2024-04</v>
+        <v>2024-05</v>
       </c>
       <c r="E11" t="str">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="F11" t="str">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="G11" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H11" t="str">
-        <v>R$ 1.320.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I11" t="str">
-        <v>7.333</v>
+        <v>12.031</v>
       </c>
       <c r="J11" t="str">
-        <v>1.1098</v>
+        <v>1.1019</v>
       </c>
       <c r="K11" t="str">
-        <v>8.139</v>
+        <v>13.258</v>
       </c>
       <c r="L11" t="str">
-        <v>29910900597</v>
+        <v>4115500247</v>
       </c>
       <c r="M11" t="str">
-        <v>~552 m (geocode da base)</v>
+        <v>~549 m (geocode da base)</v>
       </c>
       <c r="N11" t="str">
         <v>Abrir no Maps</v>
@@ -3670,40 +3670,40 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>R MARIA NOSCHESE 315</v>
+        <v>R ARAGUARI 239</v>
       </c>
       <c r="C13" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D13" t="str">
-        <v>2024-03</v>
+        <v>2025-10</v>
       </c>
       <c r="E13" t="str">
-        <v>230</v>
+        <v>190</v>
       </c>
       <c r="F13" t="str">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G13" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H13" t="str">
-        <v>R$ 1.400.000</v>
+        <v>R$ 1.900.000</v>
       </c>
       <c r="I13" t="str">
-        <v>6.087</v>
+        <v>10.000</v>
       </c>
       <c r="J13" t="str">
-        <v>1.1164</v>
+        <v>1.0190</v>
       </c>
       <c r="K13" t="str">
-        <v>6.796</v>
+        <v>10.190</v>
       </c>
       <c r="L13" t="str">
-        <v>4127700327</v>
+        <v>4108000171</v>
       </c>
       <c r="M13" t="str">
-        <v>~800 m (geocode da base)</v>
+        <v>~816 m (geocode da base)</v>
       </c>
       <c r="N13" t="str">
         <v>Abrir no Maps</v>
@@ -3726,40 +3726,40 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>R ILAMONIA 203</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 74</v>
       </c>
       <c r="C14" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-08</v>
+        <v>2024-11</v>
       </c>
       <c r="E14" t="str">
-        <v>184</v>
+        <v>247</v>
       </c>
       <c r="F14" t="str">
-        <v>170</v>
+        <v>280</v>
       </c>
       <c r="G14" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H14" t="str">
-        <v>R$ 1.500.000</v>
+        <v>R$ 1.200.000</v>
       </c>
       <c r="I14" t="str">
-        <v>8.152</v>
+        <v>4.858</v>
       </c>
       <c r="J14" t="str">
-        <v>1.0288</v>
+        <v>1.0648</v>
       </c>
       <c r="K14" t="str">
-        <v>8.387</v>
+        <v>5.173</v>
       </c>
       <c r="L14" t="str">
-        <v>4119600319</v>
+        <v>4123100104</v>
       </c>
       <c r="M14" t="str">
-        <v>~612 m (geocode da base)</v>
+        <v>~456 m (geocode da base)</v>
       </c>
       <c r="N14" t="str">
         <v>Abrir no Maps</v>
@@ -3782,40 +3782,40 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>AL DOS ARAPANES 1671</v>
+        <v>R IRAUNA 669</v>
       </c>
       <c r="C15" t="str">
         <v>Moema</v>
       </c>
       <c r="D15" t="str">
-        <v>2024-10</v>
+        <v>2024-06</v>
       </c>
       <c r="E15" t="str">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="F15" t="str">
-        <v>—</v>
+        <v>312</v>
       </c>
       <c r="G15" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H15" t="str">
-        <v>R$ 2.800.000</v>
+        <v>R$ 1.400.000</v>
       </c>
       <c r="I15" t="str">
-        <v>12.670</v>
+        <v>6.061</v>
       </c>
       <c r="J15" t="str">
-        <v>1.0697</v>
+        <v>1.0944</v>
       </c>
       <c r="K15" t="str">
-        <v>13.552</v>
+        <v>6.633</v>
       </c>
       <c r="L15" t="str">
-        <v>4122000041</v>
+        <v>4121700041</v>
       </c>
       <c r="M15" t="str">
-        <v>~901 m (geocode da base)</v>
+        <v>~617 m (geocode da base)</v>
       </c>
       <c r="N15" t="str">
         <v>Abrir no Maps</v>
@@ -3830,7 +3830,7 @@
         <v/>
       </c>
       <c r="R15" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -3838,40 +3838,40 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>R IRAUNA 550</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 77</v>
       </c>
       <c r="C16" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D16" t="str">
-        <v>2024-04</v>
+        <v>2024-03</v>
       </c>
       <c r="E16" t="str">
-        <v>279</v>
+        <v>250</v>
       </c>
       <c r="F16" t="str">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="G16" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H16" t="str">
-        <v>R$ 1.900.000</v>
+        <v>R$ 1.270.000</v>
       </c>
       <c r="I16" t="str">
-        <v>6.810</v>
+        <v>5.080</v>
       </c>
       <c r="J16" t="str">
-        <v>1.1098</v>
+        <v>1.1164</v>
       </c>
       <c r="K16" t="str">
-        <v>7.558</v>
+        <v>5.671</v>
       </c>
       <c r="L16" t="str">
-        <v>4121500180</v>
+        <v>4121400089</v>
       </c>
       <c r="M16" t="str">
-        <v>~508 m (geocode da base)</v>
+        <v>~458 m (geocode da base)</v>
       </c>
       <c r="N16" t="str">
         <v>Abrir no Maps</v>
@@ -3894,40 +3894,40 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>R ELIAS FAUSTO 34</v>
+        <v>R EMB RIBEIRO COUTO 286</v>
       </c>
       <c r="C17" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D17" t="str">
-        <v>2024-05</v>
+        <v>2025-10</v>
       </c>
       <c r="E17" t="str">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F17" t="str">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="G17" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H17" t="str">
-        <v>R$ 1.925.000</v>
+        <v>R$ 1.700.000</v>
       </c>
       <c r="I17" t="str">
-        <v>11.738</v>
+        <v>10.303</v>
       </c>
       <c r="J17" t="str">
-        <v>1.1019</v>
+        <v>1.0190</v>
       </c>
       <c r="K17" t="str">
-        <v>12.934</v>
+        <v>10.499</v>
       </c>
       <c r="L17" t="str">
-        <v>4115500239</v>
+        <v>4119700437</v>
       </c>
       <c r="M17" t="str">
-        <v>~549 m (geocode da base)</v>
+        <v>~679 m (geocode da base)</v>
       </c>
       <c r="N17" t="str">
         <v>Abrir no Maps</v>
@@ -3950,40 +3950,40 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>R CEL DAVIO ESPIRIDIAO 10</v>
+        <v>R GAIVOTA 1622</v>
       </c>
       <c r="C18" t="str">
         <v>Moema</v>
       </c>
       <c r="D18" t="str">
-        <v>2026-01</v>
+        <v>2025-03</v>
       </c>
       <c r="E18" t="str">
-        <v>275</v>
+        <v>150</v>
       </c>
       <c r="F18" t="str">
-        <v>—</v>
+        <v>187</v>
       </c>
       <c r="G18" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H18" t="str">
-        <v>R$ 3.750.000</v>
+        <v>R$ 1.650.000</v>
       </c>
       <c r="I18" t="str">
-        <v>13.636</v>
+        <v>11.000</v>
       </c>
       <c r="J18" t="str">
-        <v>1.0117</v>
+        <v>1.0488</v>
       </c>
       <c r="K18" t="str">
-        <v>13.796</v>
+        <v>11.537</v>
       </c>
       <c r="L18" t="str">
-        <v>4115700408</v>
+        <v>4119600270</v>
       </c>
       <c r="M18" t="str">
-        <v>~578 m (geocode da base)</v>
+        <v>~624 m (geocode da base)</v>
       </c>
       <c r="N18" t="str">
         <v>Abrir no Maps</v>
@@ -3998,7 +3998,7 @@
         <v/>
       </c>
       <c r="R18" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -4006,40 +4006,40 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>R ELIAS FAUSTO 40</v>
+        <v>R EMB RIBEIRO COUTO 302</v>
       </c>
       <c r="C19" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D19" t="str">
-        <v>2024-05</v>
+        <v>2025-08</v>
       </c>
       <c r="E19" t="str">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F19" t="str">
-        <v>139</v>
+        <v>264</v>
       </c>
       <c r="G19" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H19" t="str">
-        <v>R$ 1.925.000</v>
+        <v>R$ 1.540.000</v>
       </c>
       <c r="I19" t="str">
-        <v>12.031</v>
+        <v>9.935</v>
       </c>
       <c r="J19" t="str">
-        <v>1.1019</v>
+        <v>1.0288</v>
       </c>
       <c r="K19" t="str">
-        <v>13.258</v>
+        <v>10.221</v>
       </c>
       <c r="L19" t="str">
-        <v>4115500247</v>
+        <v>4119700410</v>
       </c>
       <c r="M19" t="str">
-        <v>~549 m (geocode da base)</v>
+        <v>~694 m (geocode da base)</v>
       </c>
       <c r="N19" t="str">
         <v>Abrir no Maps</v>
@@ -4062,40 +4062,40 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 476</v>
+        <v>R IRAUNA 615</v>
       </c>
       <c r="C20" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D20" t="str">
-        <v>2024-07</v>
+        <v>2024-03</v>
       </c>
       <c r="E20" t="str">
-        <v>190</v>
+        <v>140</v>
       </c>
       <c r="F20" t="str">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="G20" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H20" t="str">
-        <v>R$ 1.500.000</v>
+        <v>R$ 1.440.000</v>
       </c>
       <c r="I20" t="str">
-        <v>7.895</v>
+        <v>10.286</v>
       </c>
       <c r="J20" t="str">
-        <v>1.0879</v>
+        <v>1.1164</v>
       </c>
       <c r="K20" t="str">
-        <v>8.589</v>
+        <v>11.483</v>
       </c>
       <c r="L20" t="str">
-        <v>4127700270</v>
+        <v>4121700211</v>
       </c>
       <c r="M20" t="str">
-        <v>~789 m (geocode da base)</v>
+        <v>~569 m (geocode da base)</v>
       </c>
       <c r="N20" t="str">
         <v>Abrir no Maps</v>
@@ -4118,40 +4118,40 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>AL DOS ARAPANES 1855</v>
+        <v>R IRAUNA 655</v>
       </c>
       <c r="C21" t="str">
         <v>Moema</v>
       </c>
       <c r="D21" t="str">
-        <v>2026-04</v>
+        <v>2024-02</v>
       </c>
       <c r="E21" t="str">
-        <v>212</v>
+        <v>248</v>
       </c>
       <c r="F21" t="str">
-        <v>—</v>
+        <v>312</v>
       </c>
       <c r="G21" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H21" t="str">
-        <v>R$ 1.925.000</v>
+        <v>R$ 2.350.000</v>
       </c>
       <c r="I21" t="str">
-        <v>9.080</v>
+        <v>9.476</v>
       </c>
       <c r="J21" t="str">
-        <v>1.0030</v>
+        <v>1.1221</v>
       </c>
       <c r="K21" t="str">
-        <v>9.108</v>
+        <v>10.633</v>
       </c>
       <c r="L21" t="str">
-        <v>4127900083</v>
+        <v>4121700120</v>
       </c>
       <c r="M21" t="str">
-        <v>~956 m (geocode da base)</v>
+        <v>~604 m (geocode da base)</v>
       </c>
       <c r="N21" t="str">
         <v>Abrir no Maps</v>
@@ -4166,7 +4166,7 @@
         <v/>
       </c>
       <c r="R21" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -4174,40 +4174,40 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>R IRAUNA 916</v>
+        <v>R NOVA CIDADE 351</v>
       </c>
       <c r="C22" t="str">
-        <v>Moema</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D22" t="str">
-        <v>2024-12</v>
+        <v>2025-10</v>
       </c>
       <c r="E22" t="str">
-        <v>243</v>
+        <v>156</v>
       </c>
       <c r="F22" t="str">
-        <v>238</v>
+        <v>122</v>
       </c>
       <c r="G22" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H22" t="str">
-        <v>R$ 3.008.000</v>
+        <v>R$ 1.300.000</v>
       </c>
       <c r="I22" t="str">
-        <v>12.379</v>
+        <v>8.333</v>
       </c>
       <c r="J22" t="str">
-        <v>1.0595</v>
+        <v>1.0190</v>
       </c>
       <c r="K22" t="str">
-        <v>13.115</v>
+        <v>8.492</v>
       </c>
       <c r="L22" t="str">
-        <v>4123600263</v>
+        <v>29910100779</v>
       </c>
       <c r="M22" t="str">
-        <v>~848 m (geocode da base)</v>
+        <v>~723 m (geocode da base)</v>
       </c>
       <c r="N22" t="str">
         <v>Abrir no Maps</v>
@@ -4230,40 +4230,40 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>R ARAGUARI 239</v>
+        <v>R MARIA NOSCHESE 315</v>
       </c>
       <c r="C23" t="str">
-        <v>Vila Olímpia</v>
+        <v>não verificado</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-10</v>
+        <v>2024-03</v>
       </c>
       <c r="E23" t="str">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="F23" t="str">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G23" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H23" t="str">
-        <v>R$ 1.900.000</v>
+        <v>R$ 1.400.000</v>
       </c>
       <c r="I23" t="str">
-        <v>10.000</v>
+        <v>6.087</v>
       </c>
       <c r="J23" t="str">
-        <v>1.0190</v>
+        <v>1.1164</v>
       </c>
       <c r="K23" t="str">
-        <v>10.190</v>
+        <v>6.796</v>
       </c>
       <c r="L23" t="str">
-        <v>4108000171</v>
+        <v>4127700327</v>
       </c>
       <c r="M23" t="str">
-        <v>~816 m (geocode da base)</v>
+        <v>~800 m (geocode da base)</v>
       </c>
       <c r="N23" t="str">
         <v>Abrir no Maps</v>
@@ -4286,37 +4286,37 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>R IRAUNA 1032</v>
+        <v>AL DOS ARAPANES 1855</v>
       </c>
       <c r="C24" t="str">
         <v>Moema</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-11</v>
+        <v>2026-04</v>
       </c>
       <c r="E24" t="str">
-        <v>234</v>
+        <v>212</v>
       </c>
       <c r="F24" t="str">
-        <v>250</v>
+        <v>—</v>
       </c>
       <c r="G24" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H24" t="str">
-        <v>R$ 3.100.000</v>
+        <v>R$ 1.925.000</v>
       </c>
       <c r="I24" t="str">
-        <v>13.248</v>
+        <v>9.080</v>
       </c>
       <c r="J24" t="str">
-        <v>1.0148</v>
+        <v>1.0030</v>
       </c>
       <c r="K24" t="str">
-        <v>13.444</v>
+        <v>9.108</v>
       </c>
       <c r="L24" t="str">
-        <v>4123800084</v>
+        <v>4127900083</v>
       </c>
       <c r="M24" t="str">
         <v>~956 m (geocode da base)</v>
@@ -4334,7 +4334,7 @@
         <v/>
       </c>
       <c r="R24" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="25">
@@ -4342,40 +4342,40 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>R EMB RIBEIRO COUTO 286</v>
+        <v>AL DOS ARAPANES 1671</v>
       </c>
       <c r="C25" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-10</v>
+        <v>2024-10</v>
       </c>
       <c r="E25" t="str">
-        <v>165</v>
+        <v>221</v>
       </c>
       <c r="F25" t="str">
-        <v>272</v>
+        <v>—</v>
       </c>
       <c r="G25" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H25" t="str">
-        <v>R$ 1.700.000</v>
+        <v>R$ 2.800.000</v>
       </c>
       <c r="I25" t="str">
-        <v>10.303</v>
+        <v>12.670</v>
       </c>
       <c r="J25" t="str">
-        <v>1.0190</v>
+        <v>1.0697</v>
       </c>
       <c r="K25" t="str">
-        <v>10.499</v>
+        <v>13.552</v>
       </c>
       <c r="L25" t="str">
-        <v>4119700437</v>
+        <v>4122000041</v>
       </c>
       <c r="M25" t="str">
-        <v>~679 m (geocode da base)</v>
+        <v>~901 m (geocode da base)</v>
       </c>
       <c r="N25" t="str">
         <v>Abrir no Maps</v>
@@ -4390,7 +4390,7 @@
         <v/>
       </c>
       <c r="R25" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="26">
@@ -4398,40 +4398,40 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>R GAIVOTA 1622</v>
+        <v>AL DOS ARAPANES 1614</v>
       </c>
       <c r="C26" t="str">
         <v>Moema</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-03</v>
+        <v>2024-08</v>
       </c>
       <c r="E26" t="str">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="F26" t="str">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="G26" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H26" t="str">
-        <v>R$ 1.650.000</v>
+        <v>R$ 1.240.000</v>
       </c>
       <c r="I26" t="str">
-        <v>11.000</v>
+        <v>7.470</v>
       </c>
       <c r="J26" t="str">
-        <v>1.0488</v>
+        <v>1.0812</v>
       </c>
       <c r="K26" t="str">
-        <v>11.537</v>
+        <v>8.076</v>
       </c>
       <c r="L26" t="str">
-        <v>4119600270</v>
+        <v>4119800369</v>
       </c>
       <c r="M26" t="str">
-        <v>~624 m (geocode da base)</v>
+        <v>~891 m (geocode da base)</v>
       </c>
       <c r="N26" t="str">
         <v>Abrir no Maps</v>
@@ -4454,40 +4454,40 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>R ILAMONIA 153</v>
+        <v>AV DR CARDOSO DE MELO 379</v>
       </c>
       <c r="C27" t="str">
-        <v>Moema</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D27" t="str">
-        <v>2024-09</v>
+        <v>2025-10</v>
       </c>
       <c r="E27" t="str">
-        <v>300</v>
+        <v>95</v>
       </c>
       <c r="F27" t="str">
-        <v>277</v>
+        <v>67</v>
       </c>
       <c r="G27" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H27" t="str">
-        <v>R$ 2.000.000</v>
+        <v>R$ 1.500.000</v>
       </c>
       <c r="I27" t="str">
-        <v>6.667</v>
+        <v>15.789</v>
       </c>
       <c r="J27" t="str">
-        <v>1.0755</v>
+        <v>1.0190</v>
       </c>
       <c r="K27" t="str">
-        <v>7.170</v>
+        <v>16.090</v>
       </c>
       <c r="L27" t="str">
-        <v>4119600221</v>
+        <v>29911001189</v>
       </c>
       <c r="M27" t="str">
-        <v>~562 m (geocode da base)</v>
+        <v>~327 m (geocode da base)</v>
       </c>
       <c r="N27" t="str">
         <v>Abrir no Maps</v>
@@ -4510,40 +4510,40 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>R IRAUNA 615</v>
+        <v>R QUICABA 37</v>
       </c>
       <c r="C28" t="str">
-        <v>Moema</v>
+        <v>Vila Nova Conceição</v>
       </c>
       <c r="D28" t="str">
-        <v>2024-03</v>
+        <v>2024-04</v>
       </c>
       <c r="E28" t="str">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="F28" t="str">
-        <v>160</v>
+        <v>96</v>
       </c>
       <c r="G28" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H28" t="str">
-        <v>R$ 1.440.000</v>
+        <v>R$ 2.800.000</v>
       </c>
       <c r="I28" t="str">
-        <v>10.286</v>
+        <v>17.178</v>
       </c>
       <c r="J28" t="str">
-        <v>1.1164</v>
+        <v>1.1098</v>
       </c>
       <c r="K28" t="str">
-        <v>11.483</v>
+        <v>19.064</v>
       </c>
       <c r="L28" t="str">
-        <v>4121700211</v>
+        <v>4105700383</v>
       </c>
       <c r="M28" t="str">
-        <v>~569 m (geocode da base)</v>
+        <v>~916 m (geocode da base)</v>
       </c>
       <c r="N28" t="str">
         <v>Abrir no Maps</v>
@@ -4566,40 +4566,40 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>R IRAUNA 83</v>
+        <v>AL DOS ARAPANES 1612</v>
       </c>
       <c r="C29" t="str">
         <v>Moema</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-07</v>
+        <v>2025-03</v>
       </c>
       <c r="E29" t="str">
-        <v>340</v>
+        <v>160</v>
       </c>
       <c r="F29" t="str">
-        <v>480</v>
+        <v>224</v>
       </c>
       <c r="G29" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H29" t="str">
-        <v>R$ 1.176.125</v>
+        <v>R$ 1.870.000</v>
       </c>
       <c r="I29" t="str">
-        <v>3.459</v>
+        <v>11.688</v>
       </c>
       <c r="J29" t="str">
-        <v>1.0332</v>
+        <v>1.0488</v>
       </c>
       <c r="K29" t="str">
-        <v>3.574</v>
+        <v>12.258</v>
       </c>
       <c r="L29" t="str">
-        <v>29911800091</v>
+        <v>4119800377</v>
       </c>
       <c r="M29" t="str">
-        <v>~267 m (geocode da base)</v>
+        <v>~891 m (geocode da base)</v>
       </c>
       <c r="N29" t="str">
         <v>Abrir no Maps</v>
@@ -4622,40 +4622,40 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>R EMB RIBEIRO COUTO 302</v>
+        <v>R IRAUNA 550</v>
       </c>
       <c r="C30" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-08</v>
+        <v>2024-04</v>
       </c>
       <c r="E30" t="str">
-        <v>155</v>
+        <v>279</v>
       </c>
       <c r="F30" t="str">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="G30" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H30" t="str">
-        <v>R$ 1.540.000</v>
+        <v>R$ 1.900.000</v>
       </c>
       <c r="I30" t="str">
-        <v>9.935</v>
+        <v>6.810</v>
       </c>
       <c r="J30" t="str">
-        <v>1.0288</v>
+        <v>1.1098</v>
       </c>
       <c r="K30" t="str">
-        <v>10.221</v>
+        <v>7.558</v>
       </c>
       <c r="L30" t="str">
-        <v>4119700410</v>
+        <v>4121500180</v>
       </c>
       <c r="M30" t="str">
-        <v>~694 m (geocode da base)</v>
+        <v>~508 m (geocode da base)</v>
       </c>
       <c r="N30" t="str">
         <v>Abrir no Maps</v>
@@ -4678,40 +4678,40 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>R EMB RIBEIRO COUTO 50</v>
+        <v>R IRAUNA 916</v>
       </c>
       <c r="C31" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D31" t="str">
-        <v>2024-09</v>
+        <v>2024-12</v>
       </c>
       <c r="E31" t="str">
-        <v>320</v>
+        <v>243</v>
       </c>
       <c r="F31" t="str">
-        <v>360</v>
+        <v>238</v>
       </c>
       <c r="G31" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H31" t="str">
-        <v>R$ 2.900.000</v>
+        <v>R$ 3.008.000</v>
       </c>
       <c r="I31" t="str">
-        <v>9.063</v>
+        <v>12.379</v>
       </c>
       <c r="J31" t="str">
-        <v>1.0755</v>
+        <v>1.0595</v>
       </c>
       <c r="K31" t="str">
-        <v>9.746</v>
+        <v>13.115</v>
       </c>
       <c r="L31" t="str">
-        <v>4119500136</v>
+        <v>4123600263</v>
       </c>
       <c r="M31" t="str">
-        <v>~429 m (geocode da base)</v>
+        <v>~848 m (geocode da base)</v>
       </c>
       <c r="N31" t="str">
         <v>Abrir no Maps</v>
@@ -4734,40 +4734,40 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>R GRAUNA 86</v>
+        <v>R RIBEIRAO CLARO 684</v>
       </c>
       <c r="C32" t="str">
         <v>Vila Olímpia</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-01</v>
+        <v>2024-03</v>
       </c>
       <c r="E32" t="str">
-        <v>303</v>
+        <v>133</v>
       </c>
       <c r="F32" t="str">
-        <v>320</v>
+        <v>150</v>
       </c>
       <c r="G32" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H32" t="str">
-        <v>R$ 5.000.000</v>
+        <v>R$ 1.450.000</v>
       </c>
       <c r="I32" t="str">
-        <v>16.502</v>
+        <v>10.902</v>
       </c>
       <c r="J32" t="str">
-        <v>1.0552</v>
+        <v>1.1164</v>
       </c>
       <c r="K32" t="str">
-        <v>17.412</v>
+        <v>12.171</v>
       </c>
       <c r="L32" t="str">
-        <v>4109401836</v>
+        <v>29910900473</v>
       </c>
       <c r="M32" t="str">
-        <v>~570 m (geocode da base)</v>
+        <v>~712 m (geocode da base)</v>
       </c>
       <c r="N32" t="str">
         <v>Abrir no Maps</v>
@@ -4790,40 +4790,40 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>R NOVA CIDADE 351</v>
+        <v>R CEL DAVIO ESPIRIDIAO 10</v>
       </c>
       <c r="C33" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-10</v>
+        <v>2026-01</v>
       </c>
       <c r="E33" t="str">
-        <v>156</v>
+        <v>275</v>
       </c>
       <c r="F33" t="str">
-        <v>122</v>
+        <v>—</v>
       </c>
       <c r="G33" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H33" t="str">
-        <v>R$ 1.300.000</v>
+        <v>R$ 3.750.000</v>
       </c>
       <c r="I33" t="str">
-        <v>8.333</v>
+        <v>13.636</v>
       </c>
       <c r="J33" t="str">
-        <v>1.0190</v>
+        <v>1.0117</v>
       </c>
       <c r="K33" t="str">
-        <v>8.492</v>
+        <v>13.796</v>
       </c>
       <c r="L33" t="str">
-        <v>29910100779</v>
+        <v>4115700408</v>
       </c>
       <c r="M33" t="str">
-        <v>~723 m (geocode da base)</v>
+        <v>~578 m (geocode da base)</v>
       </c>
       <c r="N33" t="str">
         <v>Abrir no Maps</v>
@@ -4838,7 +4838,7 @@
         <v/>
       </c>
       <c r="R33" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="34">
@@ -4846,40 +4846,40 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>R DR JOSE CANDIDO DE SOUZA 542</v>
+        <v>R TUIM 229</v>
       </c>
       <c r="C34" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-09</v>
+        <v>2026-04</v>
       </c>
       <c r="E34" t="str">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="F34" t="str">
-        <v>300</v>
+        <v>—</v>
       </c>
       <c r="G34" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H34" t="str">
-        <v>R$ 1.775.000</v>
+        <v>R$ 2.450.000</v>
       </c>
       <c r="I34" t="str">
-        <v>6.526</v>
+        <v>14.848</v>
       </c>
       <c r="J34" t="str">
-        <v>1.0236</v>
+        <v>1.0030</v>
       </c>
       <c r="K34" t="str">
-        <v>6.680</v>
+        <v>14.893</v>
       </c>
       <c r="L34" t="str">
-        <v>4127800161</v>
+        <v>4108300122</v>
       </c>
       <c r="M34" t="str">
-        <v>~848 m (geocode da base)</v>
+        <v>~989 m (geocode da base)</v>
       </c>
       <c r="N34" t="str">
         <v>Abrir no Maps</v>
@@ -4894,7 +4894,7 @@
         <v/>
       </c>
       <c r="R34" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="35">
@@ -4902,40 +4902,40 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>R MARIA DE LOURDES 31</v>
+        <v>R IRAUNA 1032</v>
       </c>
       <c r="C35" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D35" t="str">
-        <v>2024-05</v>
+        <v>2025-11</v>
       </c>
       <c r="E35" t="str">
-        <v>256</v>
+        <v>234</v>
       </c>
       <c r="F35" t="str">
-        <v>315</v>
+        <v>250</v>
       </c>
       <c r="G35" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H35" t="str">
-        <v>R$ 3.300.000</v>
+        <v>R$ 3.100.000</v>
       </c>
       <c r="I35" t="str">
-        <v>12.891</v>
+        <v>13.248</v>
       </c>
       <c r="J35" t="str">
-        <v>1.1019</v>
+        <v>1.0148</v>
       </c>
       <c r="K35" t="str">
-        <v>14.205</v>
+        <v>13.444</v>
       </c>
       <c r="L35" t="str">
-        <v>4122100062</v>
+        <v>4123800084</v>
       </c>
       <c r="M35" t="str">
-        <v>~975 m (geocode da base)</v>
+        <v>~956 m (geocode da base)</v>
       </c>
       <c r="N35" t="str">
         <v>Abrir no Maps</v>
@@ -4958,40 +4958,40 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>AV DR CARDOSO DE MELO 379</v>
+        <v>R MARIA DE LOURDES 35</v>
       </c>
       <c r="C36" t="str">
-        <v>Vila Olímpia</v>
+        <v>não verificado</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-10</v>
+        <v>2024-05</v>
       </c>
       <c r="E36" t="str">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="F36" t="str">
-        <v>67</v>
+        <v>167</v>
       </c>
       <c r="G36" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H36" t="str">
-        <v>R$ 1.500.000</v>
+        <v>R$ 1.490.000</v>
       </c>
       <c r="I36" t="str">
-        <v>15.789</v>
+        <v>9.675</v>
       </c>
       <c r="J36" t="str">
-        <v>1.0190</v>
+        <v>1.1019</v>
       </c>
       <c r="K36" t="str">
-        <v>16.090</v>
+        <v>10.662</v>
       </c>
       <c r="L36" t="str">
-        <v>29911001189</v>
+        <v>4122100186</v>
       </c>
       <c r="M36" t="str">
-        <v>~327 m (geocode da base)</v>
+        <v>~975 m (geocode da base)</v>
       </c>
       <c r="N36" t="str">
         <v>Abrir no Maps</v>
@@ -5014,40 +5014,40 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>AL DOS ARAPANES 1614</v>
+        <v>R SILVANIA 65</v>
       </c>
       <c r="C37" t="str">
-        <v>Moema</v>
+        <v>não verificado</v>
       </c>
       <c r="D37" t="str">
-        <v>2024-08</v>
+        <v>2024-05</v>
       </c>
       <c r="E37" t="str">
-        <v>166</v>
+        <v>135</v>
       </c>
       <c r="F37" t="str">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="G37" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H37" t="str">
-        <v>R$ 1.240.000</v>
+        <v>R$ 2.500.000</v>
       </c>
       <c r="I37" t="str">
-        <v>7.470</v>
+        <v>18.519</v>
       </c>
       <c r="J37" t="str">
-        <v>1.0812</v>
+        <v>1.1019</v>
       </c>
       <c r="K37" t="str">
-        <v>8.076</v>
+        <v>20.406</v>
       </c>
       <c r="L37" t="str">
-        <v>4119800369</v>
+        <v>4105400177</v>
       </c>
       <c r="M37" t="str">
-        <v>~891 m (geocode da base)</v>
+        <v>~821 m (geocode da base)</v>
       </c>
       <c r="N37" t="str">
         <v>Abrir no Maps</v>
@@ -5070,40 +5070,40 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>AL DOS ARAPANES 1612</v>
+        <v>R ELIZABETH TROVAO USUI 65</v>
       </c>
       <c r="C38" t="str">
-        <v>Moema</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-03</v>
+        <v>2024-04</v>
       </c>
       <c r="E38" t="str">
-        <v>160</v>
+        <v>111</v>
       </c>
       <c r="F38" t="str">
-        <v>224</v>
+        <v>99</v>
       </c>
       <c r="G38" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H38" t="str">
-        <v>R$ 1.870.000</v>
+        <v>R$ 1.560.000</v>
       </c>
       <c r="I38" t="str">
-        <v>11.688</v>
+        <v>14.054</v>
       </c>
       <c r="J38" t="str">
-        <v>1.0488</v>
+        <v>1.1098</v>
       </c>
       <c r="K38" t="str">
-        <v>12.258</v>
+        <v>15.597</v>
       </c>
       <c r="L38" t="str">
-        <v>4119800377</v>
+        <v>29909300867</v>
       </c>
       <c r="M38" t="str">
-        <v>~891 m (geocode da base)</v>
+        <v>~644 m (geocode da base)</v>
       </c>
       <c r="N38" t="str">
         <v>Abrir no Maps</v>
@@ -5126,40 +5126,40 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
-        <v>R QUICABA 37</v>
+        <v>R ELIZABETH TROVAO USUI 55</v>
       </c>
       <c r="C39" t="str">
-        <v>Vila Nova Conceição</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D39" t="str">
-        <v>2024-04</v>
+        <v>2026-04</v>
       </c>
       <c r="E39" t="str">
-        <v>163</v>
+        <v>111</v>
       </c>
       <c r="F39" t="str">
-        <v>96</v>
+        <v>—</v>
       </c>
       <c r="G39" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H39" t="str">
-        <v>R$ 2.800.000</v>
+        <v>R$ 1.800.000</v>
       </c>
       <c r="I39" t="str">
-        <v>17.178</v>
+        <v>16.216</v>
       </c>
       <c r="J39" t="str">
-        <v>1.1098</v>
+        <v>1.0030</v>
       </c>
       <c r="K39" t="str">
-        <v>19.064</v>
+        <v>16.265</v>
       </c>
       <c r="L39" t="str">
-        <v>4105700383</v>
+        <v>29909300840</v>
       </c>
       <c r="M39" t="str">
-        <v>~916 m (geocode da base)</v>
+        <v>~644 m (geocode da base)</v>
       </c>
       <c r="N39" t="str">
         <v>Abrir no Maps</v>
@@ -5174,7 +5174,7 @@
         <v/>
       </c>
       <c r="R39" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="40">
@@ -5182,40 +5182,40 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>R RIBEIRAO CLARO 684</v>
+        <v>R ELIZABETH TROVAO USUI 64</v>
       </c>
       <c r="C40" t="str">
         <v>Vila Olímpia</v>
       </c>
       <c r="D40" t="str">
-        <v>2024-03</v>
+        <v>2025-04</v>
       </c>
       <c r="E40" t="str">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="F40" t="str">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G40" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H40" t="str">
-        <v>R$ 1.450.000</v>
+        <v>R$ 1.750.000</v>
       </c>
       <c r="I40" t="str">
-        <v>10.902</v>
+        <v>15.766</v>
       </c>
       <c r="J40" t="str">
-        <v>1.1164</v>
+        <v>1.0459</v>
       </c>
       <c r="K40" t="str">
-        <v>12.171</v>
+        <v>16.490</v>
       </c>
       <c r="L40" t="str">
-        <v>29910900473</v>
+        <v>29909300875</v>
       </c>
       <c r="M40" t="str">
-        <v>~712 m (geocode da base)</v>
+        <v>~644 m (geocode da base)</v>
       </c>
       <c r="N40" t="str">
         <v>Abrir no Maps</v>
@@ -5238,40 +5238,40 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>R TUIM 229</v>
+        <v>R MARCOS LOPES 212</v>
       </c>
       <c r="C41" t="str">
-        <v>Vila Olímpia</v>
+        <v>Vila Nova Conceição</v>
       </c>
       <c r="D41" t="str">
-        <v>2026-04</v>
+        <v>2025-10</v>
       </c>
       <c r="E41" t="str">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="F41" t="str">
-        <v>—</v>
+        <v>171</v>
       </c>
       <c r="G41" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H41" t="str">
-        <v>R$ 2.450.000</v>
+        <v>R$ 2.100.000</v>
       </c>
       <c r="I41" t="str">
-        <v>14.848</v>
+        <v>14.483</v>
       </c>
       <c r="J41" t="str">
-        <v>1.0030</v>
+        <v>1.0190</v>
       </c>
       <c r="K41" t="str">
-        <v>14.893</v>
+        <v>14.758</v>
       </c>
       <c r="L41" t="str">
-        <v>4108300122</v>
+        <v>4103000430</v>
       </c>
       <c r="M41" t="str">
-        <v>~989 m (geocode da base)</v>
+        <v>~953 m (geocode da base)</v>
       </c>
       <c r="N41" t="str">
         <v>Abrir no Maps</v>
@@ -5286,7 +5286,7 @@
         <v/>
       </c>
       <c r="R41" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -5294,40 +5294,40 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>AL JAUAPERI 1105</v>
+        <v>R MARCOS LOPES 204</v>
       </c>
       <c r="C42" t="str">
-        <v>Moema</v>
+        <v>Vila Nova Conceição</v>
       </c>
       <c r="D42" t="str">
-        <v>2026-04</v>
+        <v>2025-10</v>
       </c>
       <c r="E42" t="str">
-        <v>295</v>
+        <v>145</v>
       </c>
       <c r="F42" t="str">
-        <v>—</v>
+        <v>171</v>
       </c>
       <c r="G42" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H42" t="str">
-        <v>R$ 1.406.780</v>
+        <v>R$ 2.100.000</v>
       </c>
       <c r="I42" t="str">
-        <v>4.769</v>
+        <v>14.483</v>
       </c>
       <c r="J42" t="str">
-        <v>1.0030</v>
+        <v>1.0190</v>
       </c>
       <c r="K42" t="str">
-        <v>4.783</v>
+        <v>14.758</v>
       </c>
       <c r="L42" t="str">
-        <v>4116100919</v>
+        <v>4103000422</v>
       </c>
       <c r="M42" t="str">
-        <v>~875 m (geocode da base)</v>
+        <v>~953 m (geocode da base)</v>
       </c>
       <c r="N42" t="str">
         <v>Abrir no Maps</v>
@@ -5342,7 +5342,7 @@
         <v/>
       </c>
       <c r="R42" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -5350,40 +5350,40 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>R SILVANIA 65</v>
+        <v>R ILAMONIA 153</v>
       </c>
       <c r="C43" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D43" t="str">
-        <v>2024-05</v>
+        <v>2024-09</v>
       </c>
       <c r="E43" t="str">
-        <v>135</v>
+        <v>300</v>
       </c>
       <c r="F43" t="str">
-        <v>240</v>
+        <v>277</v>
       </c>
       <c r="G43" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H43" t="str">
-        <v>R$ 2.500.000</v>
+        <v>R$ 2.000.000</v>
       </c>
       <c r="I43" t="str">
-        <v>18.519</v>
+        <v>6.667</v>
       </c>
       <c r="J43" t="str">
-        <v>1.1019</v>
+        <v>1.0755</v>
       </c>
       <c r="K43" t="str">
-        <v>20.406</v>
+        <v>7.170</v>
       </c>
       <c r="L43" t="str">
-        <v>4105400177</v>
+        <v>4119600221</v>
       </c>
       <c r="M43" t="str">
-        <v>~821 m (geocode da base)</v>
+        <v>~562 m (geocode da base)</v>
       </c>
       <c r="N43" t="str">
         <v>Abrir no Maps</v>
@@ -5406,40 +5406,40 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>R ELIZABETH TROVAO USUI 65</v>
+        <v>R GRAUNA 86</v>
       </c>
       <c r="C44" t="str">
         <v>Vila Olímpia</v>
       </c>
       <c r="D44" t="str">
-        <v>2024-04</v>
+        <v>2025-01</v>
       </c>
       <c r="E44" t="str">
-        <v>111</v>
+        <v>303</v>
       </c>
       <c r="F44" t="str">
-        <v>99</v>
+        <v>320</v>
       </c>
       <c r="G44" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H44" t="str">
-        <v>R$ 1.560.000</v>
+        <v>R$ 5.000.000</v>
       </c>
       <c r="I44" t="str">
-        <v>14.054</v>
+        <v>16.502</v>
       </c>
       <c r="J44" t="str">
-        <v>1.1098</v>
+        <v>1.0552</v>
       </c>
       <c r="K44" t="str">
-        <v>15.597</v>
+        <v>17.412</v>
       </c>
       <c r="L44" t="str">
-        <v>29909300867</v>
+        <v>4109401836</v>
       </c>
       <c r="M44" t="str">
-        <v>~644 m (geocode da base)</v>
+        <v>~570 m (geocode da base)</v>
       </c>
       <c r="N44" t="str">
         <v>Abrir no Maps</v>
@@ -5462,40 +5462,40 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>R ELIZABETH TROVAO USUI 55</v>
+        <v>R EMB RIBEIRO COUTO 50</v>
       </c>
       <c r="C45" t="str">
-        <v>Vila Olímpia</v>
+        <v>não verificado</v>
       </c>
       <c r="D45" t="str">
-        <v>2026-04</v>
+        <v>2024-09</v>
       </c>
       <c r="E45" t="str">
-        <v>111</v>
+        <v>320</v>
       </c>
       <c r="F45" t="str">
-        <v>—</v>
+        <v>360</v>
       </c>
       <c r="G45" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H45" t="str">
-        <v>R$ 1.800.000</v>
+        <v>R$ 2.900.000</v>
       </c>
       <c r="I45" t="str">
-        <v>16.216</v>
+        <v>9.063</v>
       </c>
       <c r="J45" t="str">
-        <v>1.0030</v>
+        <v>1.0755</v>
       </c>
       <c r="K45" t="str">
-        <v>16.265</v>
+        <v>9.746</v>
       </c>
       <c r="L45" t="str">
-        <v>29909300840</v>
+        <v>4119500136</v>
       </c>
       <c r="M45" t="str">
-        <v>~644 m (geocode da base)</v>
+        <v>~429 m (geocode da base)</v>
       </c>
       <c r="N45" t="str">
         <v>Abrir no Maps</v>
@@ -5510,7 +5510,7 @@
         <v/>
       </c>
       <c r="R45" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -5518,40 +5518,40 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>R ELIZABETH TROVAO USUI 64</v>
+        <v>R MARIA DE LOURDES 31</v>
       </c>
       <c r="C46" t="str">
-        <v>Vila Olímpia</v>
+        <v>não verificado</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-04</v>
+        <v>2024-05</v>
       </c>
       <c r="E46" t="str">
-        <v>111</v>
+        <v>256</v>
       </c>
       <c r="F46" t="str">
-        <v>100</v>
+        <v>315</v>
       </c>
       <c r="G46" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H46" t="str">
-        <v>R$ 1.750.000</v>
+        <v>R$ 3.300.000</v>
       </c>
       <c r="I46" t="str">
-        <v>15.766</v>
+        <v>12.891</v>
       </c>
       <c r="J46" t="str">
-        <v>1.0459</v>
+        <v>1.1019</v>
       </c>
       <c r="K46" t="str">
-        <v>16.490</v>
+        <v>14.205</v>
       </c>
       <c r="L46" t="str">
-        <v>29909300875</v>
+        <v>4122100062</v>
       </c>
       <c r="M46" t="str">
-        <v>~644 m (geocode da base)</v>
+        <v>~975 m (geocode da base)</v>
       </c>
       <c r="N46" t="str">
         <v>Abrir no Maps</v>
@@ -5574,40 +5574,40 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>R MARIA DE LOURDES 35</v>
+        <v>R IRAUNA 83</v>
       </c>
       <c r="C47" t="str">
-        <v>não verificado</v>
+        <v>Moema</v>
       </c>
       <c r="D47" t="str">
-        <v>2024-05</v>
+        <v>2025-07</v>
       </c>
       <c r="E47" t="str">
-        <v>154</v>
+        <v>340</v>
       </c>
       <c r="F47" t="str">
-        <v>167</v>
+        <v>480</v>
       </c>
       <c r="G47" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H47" t="str">
-        <v>R$ 1.490.000</v>
+        <v>R$ 1.176.125</v>
       </c>
       <c r="I47" t="str">
-        <v>9.675</v>
+        <v>3.459</v>
       </c>
       <c r="J47" t="str">
-        <v>1.1019</v>
+        <v>1.0332</v>
       </c>
       <c r="K47" t="str">
-        <v>10.662</v>
+        <v>3.574</v>
       </c>
       <c r="L47" t="str">
-        <v>4122100186</v>
+        <v>29911800091</v>
       </c>
       <c r="M47" t="str">
-        <v>~975 m (geocode da base)</v>
+        <v>~267 m (geocode da base)</v>
       </c>
       <c r="N47" t="str">
         <v>Abrir no Maps</v>
@@ -5630,40 +5630,40 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>R MARCOS LOPES 212</v>
+        <v>R DR JOSE CANDIDO DE SOUZA 542</v>
       </c>
       <c r="C48" t="str">
-        <v>Vila Nova Conceição</v>
+        <v>não verificado</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-10</v>
+        <v>2025-09</v>
       </c>
       <c r="E48" t="str">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="F48" t="str">
-        <v>171</v>
+        <v>300</v>
       </c>
       <c r="G48" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H48" t="str">
-        <v>R$ 2.100.000</v>
+        <v>R$ 1.775.000</v>
       </c>
       <c r="I48" t="str">
-        <v>14.483</v>
+        <v>6.526</v>
       </c>
       <c r="J48" t="str">
-        <v>1.0190</v>
+        <v>1.0236</v>
       </c>
       <c r="K48" t="str">
-        <v>14.758</v>
+        <v>6.680</v>
       </c>
       <c r="L48" t="str">
-        <v>4103000430</v>
+        <v>4127800161</v>
       </c>
       <c r="M48" t="str">
-        <v>~953 m (geocode da base)</v>
+        <v>~848 m (geocode da base)</v>
       </c>
       <c r="N48" t="str">
         <v>Abrir no Maps</v>
@@ -5686,40 +5686,40 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>R MARCOS LOPES 204</v>
+        <v>R STA JUSTINA 472</v>
       </c>
       <c r="C49" t="str">
-        <v>Vila Nova Conceição</v>
+        <v>não verificado</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-10</v>
+        <v>2025-02</v>
       </c>
       <c r="E49" t="str">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="F49" t="str">
-        <v>171</v>
+        <v>125</v>
       </c>
       <c r="G49" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H49" t="str">
-        <v>R$ 2.100.000</v>
+        <v>R$ 1.150.000</v>
       </c>
       <c r="I49" t="str">
-        <v>14.483</v>
+        <v>9.583</v>
       </c>
       <c r="J49" t="str">
-        <v>1.0190</v>
+        <v>1.0511</v>
       </c>
       <c r="K49" t="str">
-        <v>14.758</v>
+        <v>10.073</v>
       </c>
       <c r="L49" t="str">
-        <v>4103000422</v>
+        <v>29906000560</v>
       </c>
       <c r="M49" t="str">
-        <v>~953 m (geocode da base)</v>
+        <v>~980 m (geocode da base)</v>
       </c>
       <c r="N49" t="str">
         <v>Abrir no Maps</v>
@@ -5742,40 +5742,40 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>AL DOS ARAPANES 1707</v>
+        <v>AL JAUAPERI 1105</v>
       </c>
       <c r="C50" t="str">
         <v>Moema</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-11</v>
+        <v>2026-04</v>
       </c>
       <c r="E50" t="str">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="F50" t="str">
-        <v>341</v>
+        <v>—</v>
       </c>
       <c r="G50" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H50" t="str">
-        <v>R$ 1.480.000</v>
+        <v>R$ 1.406.780</v>
       </c>
       <c r="I50" t="str">
-        <v>4.868</v>
+        <v>4.769</v>
       </c>
       <c r="J50" t="str">
-        <v>1.0148</v>
+        <v>1.0030</v>
       </c>
       <c r="K50" t="str">
-        <v>4.941</v>
+        <v>4.783</v>
       </c>
       <c r="L50" t="str">
-        <v>4122000203</v>
+        <v>4116100919</v>
       </c>
       <c r="M50" t="str">
-        <v>~909 m (geocode da base)</v>
+        <v>~875 m (geocode da base)</v>
       </c>
       <c r="N50" t="str">
         <v>Abrir no Maps</v>
@@ -5790,7 +5790,7 @@
         <v/>
       </c>
       <c r="R50" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="51">
@@ -5798,40 +5798,40 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>R GRAUNA 29</v>
+        <v>AL DOS ARAPANES 1707</v>
       </c>
       <c r="C51" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-05</v>
+        <v>2025-11</v>
       </c>
       <c r="E51" t="str">
-        <v>360</v>
+        <v>304</v>
       </c>
       <c r="F51" t="str">
-        <v>500</v>
+        <v>341</v>
       </c>
       <c r="G51" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H51" t="str">
-        <v>R$ 2.200.000</v>
+        <v>R$ 1.480.000</v>
       </c>
       <c r="I51" t="str">
-        <v>6.111</v>
+        <v>4.868</v>
       </c>
       <c r="J51" t="str">
-        <v>1.0431</v>
+        <v>1.0148</v>
       </c>
       <c r="K51" t="str">
-        <v>6.375</v>
+        <v>4.941</v>
       </c>
       <c r="L51" t="str">
-        <v>4107800431</v>
+        <v>4122000203</v>
       </c>
       <c r="M51" t="str">
-        <v>~581 m (geocode da base)</v>
+        <v>~909 m (geocode da base)</v>
       </c>
       <c r="N51" t="str">
         <v>Abrir no Maps</v>
@@ -5854,40 +5854,40 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>AV JACUTINGA 121</v>
+        <v>R GOMES DE CARVALHO 100</v>
       </c>
       <c r="C52" t="str">
-        <v>Moema</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D52" t="str">
-        <v>2026-03</v>
+        <v>2025-04</v>
       </c>
       <c r="E52" t="str">
-        <v>324</v>
+        <v>80</v>
       </c>
       <c r="F52" t="str">
-        <v>—</v>
+        <v>65</v>
       </c>
       <c r="G52" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H52" t="str">
-        <v>R$ 2.000.000</v>
+        <v>R$ 1.200.000</v>
       </c>
       <c r="I52" t="str">
-        <v>6.173</v>
+        <v>15.000</v>
       </c>
       <c r="J52" t="str">
-        <v>1.0050</v>
+        <v>1.0459</v>
       </c>
       <c r="K52" t="str">
-        <v>6.204</v>
+        <v>15.689</v>
       </c>
       <c r="L52" t="str">
-        <v>4108200691</v>
+        <v>29910800721</v>
       </c>
       <c r="M52" t="str">
-        <v>~889 m (geocode da base)</v>
+        <v>~958 m (geocode da base)</v>
       </c>
       <c r="N52" t="str">
         <v>Abrir no Maps</v>
@@ -5902,7 +5902,7 @@
         <v/>
       </c>
       <c r="R52" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -5910,40 +5910,40 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>R STA JUSTINA 472</v>
+        <v>R GRAUNA 29</v>
       </c>
       <c r="C53" t="str">
-        <v>não verificado</v>
+        <v>Vila Olímpia</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-02</v>
+        <v>2025-05</v>
       </c>
       <c r="E53" t="str">
-        <v>120</v>
+        <v>360</v>
       </c>
       <c r="F53" t="str">
-        <v>125</v>
+        <v>500</v>
       </c>
       <c r="G53" t="str">
         <v>casa (guia oficial)</v>
       </c>
       <c r="H53" t="str">
-        <v>R$ 1.150.000</v>
+        <v>R$ 2.200.000</v>
       </c>
       <c r="I53" t="str">
-        <v>9.583</v>
+        <v>6.111</v>
       </c>
       <c r="J53" t="str">
-        <v>1.0511</v>
+        <v>1.0431</v>
       </c>
       <c r="K53" t="str">
-        <v>10.073</v>
+        <v>6.375</v>
       </c>
       <c r="L53" t="str">
-        <v>29906000560</v>
+        <v>4107800431</v>
       </c>
       <c r="M53" t="str">
-        <v>~980 m (geocode da base)</v>
+        <v>~581 m (geocode da base)</v>
       </c>
       <c r="N53" t="str">
         <v>Abrir no Maps</v>
@@ -5966,40 +5966,40 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>R GOMES DE CARVALHO 585</v>
+        <v>AV JACUTINGA 121</v>
       </c>
       <c r="C54" t="str">
-        <v>Vila Olímpia</v>
+        <v>Moema</v>
       </c>
       <c r="D54" t="str">
-        <v>2024-01</v>
+        <v>2026-03</v>
       </c>
       <c r="E54" t="str">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="F54" t="str">
-        <v>500</v>
+        <v>—</v>
       </c>
       <c r="G54" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H54" t="str">
-        <v>R$ 5.000.000</v>
+        <v>R$ 2.000.000</v>
       </c>
       <c r="I54" t="str">
-        <v>14.881</v>
+        <v>6.173</v>
       </c>
       <c r="J54" t="str">
-        <v>1.1259</v>
+        <v>1.0050</v>
       </c>
       <c r="K54" t="str">
-        <v>16.754</v>
+        <v>6.204</v>
       </c>
       <c r="L54" t="str">
-        <v>29910100833</v>
+        <v>4108200691</v>
       </c>
       <c r="M54" t="str">
-        <v>~958 m (geocode da base)</v>
+        <v>~889 m (geocode da base)</v>
       </c>
       <c r="N54" t="str">
         <v>Abrir no Maps</v>
@@ -6014,7 +6014,7 @@
         <v/>
       </c>
       <c r="R54" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="55">
@@ -6022,7 +6022,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>R GOMES DE CARVALHO 567</v>
+        <v>R GOMES DE CARVALHO 585</v>
       </c>
       <c r="C55" t="str">
         <v>Vila Olímpia</v>
@@ -6031,28 +6031,28 @@
         <v>2024-01</v>
       </c>
       <c r="E55" t="str">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="F55" t="str">
-        <v>—</v>
+        <v>500</v>
       </c>
       <c r="G55" t="str">
-        <v>casa (provável)</v>
+        <v>casa (guia oficial)</v>
       </c>
       <c r="H55" t="str">
-        <v>R$ 6.000.000</v>
+        <v>R$ 5.000.000</v>
       </c>
       <c r="I55" t="str">
-        <v>17.143</v>
+        <v>14.881</v>
       </c>
       <c r="J55" t="str">
         <v>1.1259</v>
       </c>
       <c r="K55" t="str">
-        <v>19.301</v>
+        <v>16.754</v>
       </c>
       <c r="L55" t="str">
-        <v>29910100221</v>
+        <v>29910100833</v>
       </c>
       <c r="M55" t="str">
         <v>~958 m (geocode da base)</v>
@@ -6070,7 +6070,7 @@
         <v/>
       </c>
       <c r="R55" t="str">
-        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -6078,37 +6078,37 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>R GOMES DE CARVALHO 100</v>
+        <v>R GOMES DE CARVALHO 567</v>
       </c>
       <c r="C56" t="str">
         <v>Vila Olímpia</v>
       </c>
       <c r="D56" t="str">
-        <v>2025-04</v>
+        <v>2024-01</v>
       </c>
       <c r="E56" t="str">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="F56" t="str">
-        <v>65</v>
+        <v>—</v>
       </c>
       <c r="G56" t="str">
-        <v>casa (guia oficial)</v>
+        <v>casa (provável)</v>
       </c>
       <c r="H56" t="str">
-        <v>R$ 1.200.000</v>
+        <v>R$ 6.000.000</v>
       </c>
       <c r="I56" t="str">
-        <v>15.000</v>
+        <v>17.143</v>
       </c>
       <c r="J56" t="str">
-        <v>1.0459</v>
+        <v>1.1259</v>
       </c>
       <c r="K56" t="str">
-        <v>15.689</v>
+        <v>19.301</v>
       </c>
       <c r="L56" t="str">
-        <v>29910800721</v>
+        <v>29910100221</v>
       </c>
       <c r="M56" t="str">
         <v>~958 m (geocode da base)</v>
@@ -6126,7 +6126,7 @@
         <v/>
       </c>
       <c r="R56" t="str">
-        <v/>
+        <v>PRIORIDADE: venda 2026 sem guia pública — confirmar tipologia</v>
       </c>
     </row>
     <row r="57">

</xml_diff>